<commit_message>
feat(automotive): rebuild telltale Excel with 40 telltales from official FMVSS/UN/ISO sources
Agent-Logs-Url: https://github.com/mmandalapu30/Design-System-Regulations/sessions/5f307eb9-de33-41db-bdb0-c33d39c0fe80

Co-authored-by: mmandalapu30 <268487919+mmandalapu30@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/docs/telltale-design-requirements.xlsx
+++ b/docs/telltale-design-requirements.xlsx
@@ -26,17 +26,20 @@
       <scheme val="minor"/>
     </font>
     <font>
+      <name val="Calibri"/>
       <b val="1"/>
       <color rgb="00FFFFFF"/>
-      <sz val="10"/>
-    </font>
-    <font>
       <sz val="9"/>
     </font>
     <font>
+      <name val="Calibri"/>
+      <sz val="8"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
       <i val="1"/>
       <color rgb="00555555"/>
-      <sz val="8"/>
+      <sz val="7"/>
     </font>
   </fonts>
   <fills count="5">
@@ -48,12 +51,12 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="001AAEAE"/>
+        <fgColor rgb="001A6E8E"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00E8F8F8"/>
+        <fgColor rgb="00E6F3F7"/>
       </patternFill>
     </fill>
     <fill>
@@ -105,7 +108,9 @@
     <xf numFmtId="0" fontId="2" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -191,7 +196,7 @@
       <row>1</row>
       <rowOff>0</rowOff>
     </from>
-    <ext cx="762000" cy="762000"/>
+    <ext cx="685800" cy="685800"/>
     <pic>
       <nvPicPr>
         <cNvPr id="1" name="Image 1" descr="Picture"/>
@@ -216,7 +221,7 @@
       <row>2</row>
       <rowOff>0</rowOff>
     </from>
-    <ext cx="762000" cy="762000"/>
+    <ext cx="685800" cy="685800"/>
     <pic>
       <nvPicPr>
         <cNvPr id="2" name="Image 2" descr="Picture"/>
@@ -241,7 +246,7 @@
       <row>3</row>
       <rowOff>0</rowOff>
     </from>
-    <ext cx="762000" cy="762000"/>
+    <ext cx="685800" cy="685800"/>
     <pic>
       <nvPicPr>
         <cNvPr id="3" name="Image 3" descr="Picture"/>
@@ -266,7 +271,7 @@
       <row>4</row>
       <rowOff>0</rowOff>
     </from>
-    <ext cx="762000" cy="762000"/>
+    <ext cx="685800" cy="685800"/>
     <pic>
       <nvPicPr>
         <cNvPr id="4" name="Image 4" descr="Picture"/>
@@ -291,7 +296,7 @@
       <row>5</row>
       <rowOff>0</rowOff>
     </from>
-    <ext cx="762000" cy="762000"/>
+    <ext cx="685800" cy="685800"/>
     <pic>
       <nvPicPr>
         <cNvPr id="5" name="Image 5" descr="Picture"/>
@@ -316,7 +321,7 @@
       <row>6</row>
       <rowOff>0</rowOff>
     </from>
-    <ext cx="762000" cy="762000"/>
+    <ext cx="685800" cy="685800"/>
     <pic>
       <nvPicPr>
         <cNvPr id="6" name="Image 6" descr="Picture"/>
@@ -341,7 +346,7 @@
       <row>7</row>
       <rowOff>0</rowOff>
     </from>
-    <ext cx="762000" cy="762000"/>
+    <ext cx="685800" cy="685800"/>
     <pic>
       <nvPicPr>
         <cNvPr id="7" name="Image 7" descr="Picture"/>
@@ -366,7 +371,7 @@
       <row>8</row>
       <rowOff>0</rowOff>
     </from>
-    <ext cx="762000" cy="762000"/>
+    <ext cx="685800" cy="685800"/>
     <pic>
       <nvPicPr>
         <cNvPr id="8" name="Image 8" descr="Picture"/>
@@ -391,7 +396,7 @@
       <row>9</row>
       <rowOff>0</rowOff>
     </from>
-    <ext cx="762000" cy="762000"/>
+    <ext cx="685800" cy="685800"/>
     <pic>
       <nvPicPr>
         <cNvPr id="9" name="Image 9" descr="Picture"/>
@@ -416,7 +421,7 @@
       <row>10</row>
       <rowOff>0</rowOff>
     </from>
-    <ext cx="762000" cy="762000"/>
+    <ext cx="685800" cy="685800"/>
     <pic>
       <nvPicPr>
         <cNvPr id="10" name="Image 10" descr="Picture"/>
@@ -441,7 +446,7 @@
       <row>11</row>
       <rowOff>0</rowOff>
     </from>
-    <ext cx="762000" cy="762000"/>
+    <ext cx="685800" cy="685800"/>
     <pic>
       <nvPicPr>
         <cNvPr id="11" name="Image 11" descr="Picture"/>
@@ -466,7 +471,7 @@
       <row>12</row>
       <rowOff>0</rowOff>
     </from>
-    <ext cx="762000" cy="762000"/>
+    <ext cx="685800" cy="685800"/>
     <pic>
       <nvPicPr>
         <cNvPr id="12" name="Image 12" descr="Picture"/>
@@ -474,6 +479,706 @@
       </nvPicPr>
       <blipFill>
         <a:blip cstate="print" r:embed="rId12"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>0</col>
+      <colOff>0</colOff>
+      <row>13</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="685800" cy="685800"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="13" name="Image 13" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip cstate="print" r:embed="rId13"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>0</col>
+      <colOff>0</colOff>
+      <row>14</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="685800" cy="685800"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="14" name="Image 14" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip cstate="print" r:embed="rId14"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>0</col>
+      <colOff>0</colOff>
+      <row>15</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="685800" cy="685800"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="15" name="Image 15" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip cstate="print" r:embed="rId15"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>0</col>
+      <colOff>0</colOff>
+      <row>16</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="685800" cy="685800"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="16" name="Image 16" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip cstate="print" r:embed="rId16"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>0</col>
+      <colOff>0</colOff>
+      <row>17</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="685800" cy="685800"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="17" name="Image 17" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip cstate="print" r:embed="rId17"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>0</col>
+      <colOff>0</colOff>
+      <row>18</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="685800" cy="685800"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="18" name="Image 18" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip cstate="print" r:embed="rId18"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>0</col>
+      <colOff>0</colOff>
+      <row>19</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="685800" cy="685800"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="19" name="Image 19" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip cstate="print" r:embed="rId19"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>0</col>
+      <colOff>0</colOff>
+      <row>20</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="685800" cy="685800"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="20" name="Image 20" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip cstate="print" r:embed="rId20"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>0</col>
+      <colOff>0</colOff>
+      <row>21</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="685800" cy="685800"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="21" name="Image 21" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip cstate="print" r:embed="rId21"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>0</col>
+      <colOff>0</colOff>
+      <row>22</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="685800" cy="685800"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="22" name="Image 22" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip cstate="print" r:embed="rId22"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>0</col>
+      <colOff>0</colOff>
+      <row>23</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="685800" cy="685800"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="23" name="Image 23" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip cstate="print" r:embed="rId23"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>0</col>
+      <colOff>0</colOff>
+      <row>24</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="685800" cy="685800"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="24" name="Image 24" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip cstate="print" r:embed="rId24"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>0</col>
+      <colOff>0</colOff>
+      <row>25</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="685800" cy="685800"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="25" name="Image 25" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip cstate="print" r:embed="rId25"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>0</col>
+      <colOff>0</colOff>
+      <row>26</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="685800" cy="685800"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="26" name="Image 26" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip cstate="print" r:embed="rId26"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>0</col>
+      <colOff>0</colOff>
+      <row>27</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="685800" cy="685800"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="27" name="Image 27" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip cstate="print" r:embed="rId27"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>0</col>
+      <colOff>0</colOff>
+      <row>28</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="685800" cy="685800"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="28" name="Image 28" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip cstate="print" r:embed="rId28"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>0</col>
+      <colOff>0</colOff>
+      <row>29</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="685800" cy="685800"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="29" name="Image 29" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip cstate="print" r:embed="rId29"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>0</col>
+      <colOff>0</colOff>
+      <row>30</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="685800" cy="685800"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="30" name="Image 30" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip cstate="print" r:embed="rId30"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>0</col>
+      <colOff>0</colOff>
+      <row>31</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="685800" cy="685800"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="31" name="Image 31" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip cstate="print" r:embed="rId31"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>0</col>
+      <colOff>0</colOff>
+      <row>32</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="685800" cy="685800"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="32" name="Image 32" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip cstate="print" r:embed="rId32"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>0</col>
+      <colOff>0</colOff>
+      <row>33</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="685800" cy="685800"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="33" name="Image 33" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip cstate="print" r:embed="rId33"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>0</col>
+      <colOff>0</colOff>
+      <row>34</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="685800" cy="685800"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="34" name="Image 34" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip cstate="print" r:embed="rId34"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>0</col>
+      <colOff>0</colOff>
+      <row>35</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="685800" cy="685800"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="35" name="Image 35" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip cstate="print" r:embed="rId35"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>0</col>
+      <colOff>0</colOff>
+      <row>36</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="685800" cy="685800"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="36" name="Image 36" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip cstate="print" r:embed="rId36"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>0</col>
+      <colOff>0</colOff>
+      <row>37</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="685800" cy="685800"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="37" name="Image 37" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip cstate="print" r:embed="rId37"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>0</col>
+      <colOff>0</colOff>
+      <row>38</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="685800" cy="685800"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="38" name="Image 38" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip cstate="print" r:embed="rId38"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>0</col>
+      <colOff>0</colOff>
+      <row>39</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="685800" cy="685800"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="39" name="Image 39" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip cstate="print" r:embed="rId39"/>
+        <a:stretch>
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>0</col>
+      <colOff>0</colOff>
+      <row>40</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="685800" cy="685800"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="40" name="Image 40" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip cstate="print" r:embed="rId40"/>
         <a:stretch>
           <a:fillRect/>
         </a:stretch>
@@ -776,29 +1481,30 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:N15"/>
+  <dimension ref="A1:N44"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="18" customWidth="1" min="1" max="1"/>
-    <col width="16" customWidth="1" min="2" max="2"/>
-    <col width="26" customWidth="1" min="3" max="3"/>
-    <col width="14" customWidth="1" min="4" max="4"/>
+    <col width="14" customWidth="1" min="1" max="1"/>
+    <col width="22" customWidth="1" min="2" max="2"/>
+    <col width="28" customWidth="1" min="3" max="3"/>
+    <col width="22" customWidth="1" min="4" max="4"/>
     <col width="14" customWidth="1" min="5" max="5"/>
-    <col width="16" customWidth="1" min="6" max="6"/>
-    <col width="16" customWidth="1" min="7" max="7"/>
-    <col width="10" customWidth="1" min="8" max="8"/>
+    <col width="20" customWidth="1" min="6" max="6"/>
+    <col width="22" customWidth="1" min="7" max="7"/>
+    <col width="12" customWidth="1" min="8" max="8"/>
     <col width="36" customWidth="1" min="9" max="9"/>
-    <col width="32" customWidth="1" min="10" max="10"/>
-    <col width="32" customWidth="1" min="11" max="11"/>
-    <col width="26" customWidth="1" min="12" max="12"/>
-    <col width="45" customWidth="1" min="13" max="13"/>
-    <col width="20" customWidth="1" min="14" max="14"/>
+    <col width="30" customWidth="1" min="10" max="10"/>
+    <col width="30" customWidth="1" min="11" max="11"/>
+    <col width="28" customWidth="1" min="12" max="12"/>
+    <col width="50" customWidth="1" min="13" max="13"/>
+    <col width="22" customWidth="1" min="14" max="14"/>
   </cols>
   <sheetData>
-    <row r="1" ht="48" customHeight="1">
+    <row r="1" ht="52" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
-          <t>Telltale</t>
+          <t>Telltale
+(Symbol)</t>
         </is>
       </c>
       <c r="B1" s="1" t="inlineStr">
@@ -808,7 +1514,8 @@
       </c>
       <c r="C1" s="1" t="inlineStr">
         <is>
-          <t>US Requirements</t>
+          <t>US Requirements
+(FMVSS)</t>
         </is>
       </c>
       <c r="D1" s="1" t="inlineStr">
@@ -823,7 +1530,7 @@
       </c>
       <c r="F1" s="1" t="inlineStr">
         <is>
-          <t>ISO</t>
+          <t>ISO Reference</t>
         </is>
       </c>
       <c r="G1" s="1" t="inlineStr">
@@ -845,12 +1552,14 @@
       </c>
       <c r="J1" s="1" t="inlineStr">
         <is>
-          <t>Brightness</t>
+          <t>Brightness
+Requirements</t>
         </is>
       </c>
       <c r="K1" s="1" t="inlineStr">
         <is>
-          <t>Contrast</t>
+          <t>Contrast
+Requirements</t>
         </is>
       </c>
       <c r="L1" s="1" t="inlineStr">
@@ -874,31 +1583,30 @@
       <c r="A2" s="2" t="inlineStr"/>
       <c r="B2" s="3" t="inlineStr">
         <is>
-          <t>Turn Signal</t>
+          <t>Direction Indicator (Turn Signal)</t>
         </is>
       </c>
       <c r="C2" s="3" t="inlineStr">
         <is>
-          <t>Direct – FMVSS 101
-Indirect – FMVSS 108</t>
+          <t>Direct – FMVSS 101 (49 CFR 571.101), Table 1, Item 1
+Indirect – FMVSS 108 (49 CFR 571.108)</t>
         </is>
       </c>
       <c r="D2" s="3" t="inlineStr">
         <is>
-          <t>R48</t>
+          <t>UN R48 (Rev.6), Annex 5, Item 1
+UN R121, Table 1, Row 1</t>
         </is>
       </c>
       <c r="E2" s="3" t="inlineStr"/>
       <c r="F2" s="3" t="inlineStr">
         <is>
-          <t>ISO 7000-0256</t>
+          <t>ISO 2575:2021, Symbol 7000-0256</t>
         </is>
       </c>
       <c r="G2" s="3" t="inlineStr">
         <is>
-          <t>SAE J2395
-SAE J1005
-ISO 2575</t>
+          <t>ISO 2575:2021 Cl. 5.2: minimum symbol height 5 mm at design eye point. SAE J1005: symbol ≥3.2 mm; text/numerals ≥4.8 mm. FMVSS 101 S5.3: legible at 76 cm viewing distance.</t>
         </is>
       </c>
       <c r="H2" s="3" t="inlineStr">
@@ -908,30 +1616,27 @@
       </c>
       <c r="I2" s="3" t="inlineStr">
         <is>
-          <t>Two opposing arrows. Icon must be filled in, no outline. Illumination should be uniform across the telltale, with no uneven brightness or dim spots.</t>
+          <t>Two opposing arrows (left and right). Symbol must be filled (solid), not outline only. Illumination uniform across the symbol with no dim spots. Flash rate 60–120 times/min per FMVSS 108 S7.10.</t>
         </is>
       </c>
       <c r="J2" s="3" t="inlineStr">
         <is>
-          <t>SAE J387 – minimum luminance of 2.0 cd/m²; maximum of 100 cd/m² to prevent glare at night</t>
+          <t>SAE J387 / ECE R121 Annex 4: minimum luminance 2 cd/m² (night), max 100 cd/m² (to prevent glare). Daytime: 100–1 000 cd/m².</t>
         </is>
       </c>
       <c r="K2" s="3" t="inlineStr">
         <is>
-          <t>SAE J2402 – at least 3:1 for daytime and 4.5:1 or higher for nighttime</t>
+          <t>SAE J2402: ≥3:1 luminance contrast during day; ≥4.5:1 during night. Symbol-to-background ratio.</t>
         </is>
       </c>
       <c r="L2" s="3" t="inlineStr">
         <is>
-          <t>Within the driver's primary field of view</t>
+          <t>Within the driver's primary field of view (FMVSS 101 S5.1). Visible without head movement. Not obscured by steering wheel.</t>
         </is>
       </c>
       <c r="M2" s="3" t="inlineStr">
         <is>
-          <t>The telltale must flash in sync with the vehicle's exterior turn signal lamps at a rate of 60–120 flashes per minute.
-If an exterior lamp fails, the telltale must flash at a distinctly different rate (usually faster).
-During hazard light activation, both arrows must flash together in sync with the exterior lights.
-May include subtle animation or fade-in effects if compliant with brightness and timing requirements.</t>
+          <t>Flashes in synchrony with exterior turn signal lamps at 60–120 flashes/min (FMVSS 108 S7.10.1). If an exterior lamp fails, flash rate doubles (≥120/min) per FMVSS 108 S7.10.2. During hazard operation both arrows flash simultaneously. May include fade/animation if brightness and timing remain compliant.</t>
         </is>
       </c>
       <c r="N2" s="3" t="inlineStr"/>
@@ -940,62 +1645,60 @@
       <c r="A3" s="4" t="inlineStr"/>
       <c r="B3" s="5" t="inlineStr">
         <is>
-          <t>MIL – Check Engine</t>
+          <t>High Beam Headlamp</t>
         </is>
       </c>
       <c r="C3" s="5" t="inlineStr">
         <is>
-          <t>Direct – FMVSS 101
-Indirect – SAE J1979 (OBD-II protocols)</t>
+          <t>Direct – FMVSS 101, Table 1, Item 4
+Indirect – FMVSS 108 (49 CFR 571.108)</t>
         </is>
       </c>
       <c r="D3" s="5" t="inlineStr">
         <is>
-          <t>R83</t>
+          <t>UN R48, Annex 5, Item 4
+UN R121, Table 1</t>
         </is>
       </c>
       <c r="E3" s="5" t="inlineStr"/>
       <c r="F3" s="5" t="inlineStr">
         <is>
-          <t>ISO 7000-0653</t>
+          <t>ISO 2575:2021, Symbol 7000-0053</t>
         </is>
       </c>
       <c r="G3" s="5" t="inlineStr">
         <is>
-          <t>SAE J2395
-SAE J1005
-ISO 2575</t>
+          <t>ISO 2575:2021 Cl. 5.2: minimum symbol height 5 mm at design eye point. SAE J1005: symbol ≥3.2 mm; text/numerals ≥4.8 mm. FMVSS 101 S5.3: legible at 76 cm viewing distance.</t>
         </is>
       </c>
       <c r="H3" s="5" t="inlineStr">
         <is>
-          <t>Amber</t>
+          <t>Blue</t>
         </is>
       </c>
       <c r="I3" s="5" t="inlineStr">
         <is>
-          <t>Symbol can be an outline and is not required to be filled in. May use the text "CHECK ENGINE" or equivalent wording, as long as it adheres to FMVSS 101 readability and visibility requirements.</t>
+          <t>Filled symbol (headlamp lens with parallel horizontal rays projecting forward). Must not be outlined only.</t>
         </is>
       </c>
       <c r="J3" s="5" t="inlineStr">
         <is>
-          <t>SAE J387 – minimum luminance of 2.0 cd/m²; maximum of 100 cd/m² to prevent glare at night</t>
+          <t>SAE J387 / ECE R121 Annex 4: minimum luminance 2 cd/m² (night), max 100 cd/m² (to prevent glare). Daytime: 100–1 000 cd/m².</t>
         </is>
       </c>
       <c r="K3" s="5" t="inlineStr">
         <is>
-          <t>SAE J2402 – at least 3:1 for daytime and 4.5:1 or higher for nighttime</t>
+          <t>SAE J2402: ≥3:1 luminance contrast during day; ≥4.5:1 during night. Symbol-to-background ratio.</t>
         </is>
       </c>
       <c r="L3" s="5" t="inlineStr">
         <is>
-          <t>Within the driver's primary field of view</t>
+          <t>Within the driver's primary field of view (FMVSS 101 S5.1). Visible without head movement. Not obscured by steering wheel.</t>
         </is>
       </c>
       <c r="M3" s="5" t="inlineStr">
         <is>
-          <t>Steady Light: Indicates a less severe fault that needs attention soon (e.g., emissions-related issue).
-Flashing Light: Indicates a serious fault, such as a misfire, which could cause damage to the catalytic converter or other components. Immediate action is required.</t>
+          <t>Illuminates when upper (high) beam headlamps are on. Extinguishes immediately on switching to low beam or when headlamps are turned off. Also illuminates during "flash-to-pass" activation (FMVSS 108 S7.7.1.1).</t>
         </is>
       </c>
       <c r="N3" s="5" t="inlineStr"/>
@@ -1004,31 +1707,30 @@
       <c r="A4" s="2" t="inlineStr"/>
       <c r="B4" s="3" t="inlineStr">
         <is>
-          <t>Position Lights</t>
+          <t>Low Beam Headlamp</t>
         </is>
       </c>
       <c r="C4" s="3" t="inlineStr">
         <is>
-          <t>Direct – FMVSS 101
-Indirect – FMVSS 108, 111, 135</t>
+          <t>Direct – FMVSS 101, Table 2 (voluntary)
+Indirect – FMVSS 108 (49 CFR 571.108)</t>
         </is>
       </c>
       <c r="D4" s="3" t="inlineStr">
         <is>
-          <t>R48</t>
+          <t>UN R48, Annex 5
+UN R121, Table 1</t>
         </is>
       </c>
       <c r="E4" s="3" t="inlineStr"/>
       <c r="F4" s="3" t="inlineStr">
         <is>
-          <t>ISO 7000-0257</t>
+          <t>ISO 2575:2021, Symbol 7000-0052</t>
         </is>
       </c>
       <c r="G4" s="3" t="inlineStr">
         <is>
-          <t>SAE J2395
-SAE J1005
-ISO 2575</t>
+          <t>ISO 2575:2021 Cl. 5.2: minimum symbol height 5 mm at design eye point. SAE J1005: symbol ≥3.2 mm; text/numerals ≥4.8 mm. FMVSS 101 S5.3: legible at 76 cm viewing distance.</t>
         </is>
       </c>
       <c r="H4" s="3" t="inlineStr">
@@ -1038,27 +1740,27 @@
       </c>
       <c r="I4" s="3" t="inlineStr">
         <is>
-          <t>The symbol can either be an outline or filled.</t>
+          <t>Filled headlamp symbol with rays angled downward and to the left (or shield). Must be distinguishable from the high beam symbol.</t>
         </is>
       </c>
       <c r="J4" s="3" t="inlineStr">
         <is>
-          <t>SAE J387 – minimum luminance of 2.0 cd/m²; maximum of 100 cd/m² to prevent glare at night</t>
+          <t>SAE J387 / ECE R121 Annex 4: minimum luminance 2 cd/m² (night), max 100 cd/m² (to prevent glare). Daytime: 100–1 000 cd/m².</t>
         </is>
       </c>
       <c r="K4" s="3" t="inlineStr">
         <is>
-          <t>SAE J2402 – at least 3:1 for daytime and 4.5:1 or higher for nighttime</t>
+          <t>SAE J2402: ≥3:1 luminance contrast during day; ≥4.5:1 during night. Symbol-to-background ratio.</t>
         </is>
       </c>
       <c r="L4" s="3" t="inlineStr">
         <is>
-          <t>Within the driver's primary field of view</t>
+          <t>Within the driver's primary field of view (FMVSS 101 S5.1). Visible without head movement. Not obscured by steering wheel.</t>
         </is>
       </c>
       <c r="M4" s="3" t="inlineStr">
         <is>
-          <t>Illuminates whenever the position (parking) lights are active, regardless of whether the headlights are on or off.</t>
+          <t>Illuminates when low (dipped) beam headlamps are activated. Extinguishes when headlamps are turned off or switched to high beam (high beam telltale then activates).</t>
         </is>
       </c>
       <c r="N4" s="3" t="inlineStr"/>
@@ -1067,62 +1769,60 @@
       <c r="A5" s="4" t="inlineStr"/>
       <c r="B5" s="5" t="inlineStr">
         <is>
-          <t>Tire Pressure</t>
+          <t>Position (Parking) Lamps</t>
         </is>
       </c>
       <c r="C5" s="5" t="inlineStr">
         <is>
-          <t>Direct – FMVSS 101
-Indirect – FMVSS 138</t>
+          <t>Direct – FMVSS 101, Table 2 (voluntary)
+Indirect – FMVSS 108, 111, 135 (49 CFR 571.108/111/135)</t>
         </is>
       </c>
       <c r="D5" s="5" t="inlineStr">
         <is>
-          <t>R141</t>
+          <t>UN R48, Annex 5
+UN R121, Table 1</t>
         </is>
       </c>
       <c r="E5" s="5" t="inlineStr"/>
       <c r="F5" s="5" t="inlineStr">
         <is>
-          <t>ISO 7000-1109</t>
+          <t>ISO 2575:2021, Symbol 7000-0257</t>
         </is>
       </c>
       <c r="G5" s="5" t="inlineStr">
         <is>
-          <t>SAE J2395
-SAE J1005
-ISO 2575</t>
+          <t>ISO 2575:2021 Cl. 5.2: minimum symbol height 5 mm at design eye point. SAE J1005: symbol ≥3.2 mm; text/numerals ≥4.8 mm. FMVSS 101 S5.3: legible at 76 cm viewing distance.</t>
         </is>
       </c>
       <c r="H5" s="5" t="inlineStr">
         <is>
-          <t>Amber</t>
+          <t>Green</t>
         </is>
       </c>
       <c r="I5" s="5" t="inlineStr">
         <is>
-          <t>Symbol must be filled-in, not just an outline.</t>
+          <t>Symbol may be outline or filled. Represents sidelights / parking lamps.</t>
         </is>
       </c>
       <c r="J5" s="5" t="inlineStr">
         <is>
-          <t>SAE J387 – minimum luminance of 2.0 cd/m²; maximum of 100 cd/m² to prevent glare at night</t>
+          <t>SAE J387 / ECE R121 Annex 4: minimum luminance 2 cd/m² (night), max 100 cd/m² (to prevent glare). Daytime: 100–1 000 cd/m².</t>
         </is>
       </c>
       <c r="K5" s="5" t="inlineStr">
         <is>
-          <t>SAE J2402 – at least 3:1 for daytime and 4.5:1 or higher for nighttime</t>
+          <t>SAE J2402: ≥3:1 luminance contrast during day; ≥4.5:1 during night. Symbol-to-background ratio.</t>
         </is>
       </c>
       <c r="L5" s="5" t="inlineStr">
         <is>
-          <t>Within the driver's primary field of view</t>
+          <t>Within the driver's primary field of view (FMVSS 101 S5.1). Visible without head movement. Not obscured by steering wheel.</t>
         </is>
       </c>
       <c r="M5" s="5" t="inlineStr">
         <is>
-          <t>A steady light signals a low tire pressure.
-A flashing light typically signals a fault in the TPMS system itself, such as a sensor failure.</t>
+          <t>Illuminates whenever parking/position lamps are active, regardless of whether full headlamps are on. Extinguishes when position lamps are turned off.</t>
         </is>
       </c>
       <c r="N5" s="5" t="inlineStr"/>
@@ -1131,61 +1831,60 @@
       <c r="A6" s="2" t="inlineStr"/>
       <c r="B6" s="3" t="inlineStr">
         <is>
-          <t>High Beam</t>
+          <t>Front Fog Lamp</t>
         </is>
       </c>
       <c r="C6" s="3" t="inlineStr">
         <is>
-          <t>Direct – FMVSS 101
-Indirect – FMVSS 108</t>
+          <t>Direct – FMVSS 101, Table 2 (voluntary)
+Indirect – FMVSS 108 (49 CFR 571.108)</t>
         </is>
       </c>
       <c r="D6" s="3" t="inlineStr">
         <is>
-          <t>R48</t>
+          <t>UN R48, Annex 5
+UN R121, Table 1, Row 12</t>
         </is>
       </c>
       <c r="E6" s="3" t="inlineStr"/>
       <c r="F6" s="3" t="inlineStr">
         <is>
-          <t>ISO 7000-0053</t>
+          <t>ISO 2575:2021, Symbol 7000-2048</t>
         </is>
       </c>
       <c r="G6" s="3" t="inlineStr">
         <is>
-          <t>SAE J2395
-SAE J1005
-ISO 2575</t>
+          <t>ISO 2575:2021 Cl. 5.2: minimum symbol height 5 mm at design eye point. SAE J1005: symbol ≥3.2 mm; text/numerals ≥4.8 mm. FMVSS 101 S5.3: legible at 76 cm viewing distance.</t>
         </is>
       </c>
       <c r="H6" s="3" t="inlineStr">
         <is>
-          <t>Blue</t>
+          <t>Green</t>
         </is>
       </c>
       <c r="I6" s="3" t="inlineStr">
         <is>
-          <t>Symbol must be filled-in, not an outline.</t>
+          <t>Filled symbol: headlamp lens with rays angled through downward-slanted parallel lines representing fog.</t>
         </is>
       </c>
       <c r="J6" s="3" t="inlineStr">
         <is>
-          <t>SAE J387 – minimum luminance of 2.0 cd/m²; maximum of 100 cd/m² to prevent glare at night</t>
+          <t>SAE J387 / ECE R121 Annex 4: minimum luminance 2 cd/m² (night), max 100 cd/m² (to prevent glare). Daytime: 100–1 000 cd/m².</t>
         </is>
       </c>
       <c r="K6" s="3" t="inlineStr">
         <is>
-          <t>SAE J2402 – at least 3:1 for daytime and 4.5:1 or higher for nighttime</t>
+          <t>SAE J2402: ≥3:1 luminance contrast during day; ≥4.5:1 during night. Symbol-to-background ratio.</t>
         </is>
       </c>
       <c r="L6" s="3" t="inlineStr">
         <is>
-          <t>Within the driver's primary field of view</t>
+          <t>Within the driver's primary field of view (FMVSS 101 S5.1). Visible without head movement. Not obscured by steering wheel.</t>
         </is>
       </c>
       <c r="M6" s="3" t="inlineStr">
         <is>
-          <t>The telltale illuminates when the high beam headlamps are on. It must turn off when high beams are switched off or when switched to low beam. Also flashes with "flash to pass".</t>
+          <t>Illuminates when front fog lamps are switched on. Extinguishes when fog lamps are switched off. On vehicles with integrated lighting, front fogs may auto-deactivate when high beams are engaged (design-dependent).</t>
         </is>
       </c>
       <c r="N6" s="3" t="inlineStr"/>
@@ -1194,31 +1893,30 @@
       <c r="A7" s="4" t="inlineStr"/>
       <c r="B7" s="5" t="inlineStr">
         <is>
-          <t>ESC Off</t>
+          <t>Rear Fog Lamp</t>
         </is>
       </c>
       <c r="C7" s="5" t="inlineStr">
         <is>
-          <t>Direct – FMVSS 101
-Indirect – FMVSS 108 &amp; 136</t>
+          <t>Direct – FMVSS 101, Table 2 (voluntary)
+Indirect – FMVSS 108 (49 CFR 571.108)</t>
         </is>
       </c>
       <c r="D7" s="5" t="inlineStr">
         <is>
-          <t>R140</t>
+          <t>UN R48, Annex 5
+UN R121, Table 1, Row 13</t>
         </is>
       </c>
       <c r="E7" s="5" t="inlineStr"/>
       <c r="F7" s="5" t="inlineStr">
         <is>
-          <t>ISO 7000-0801</t>
+          <t>ISO 2575:2021, Symbol 7000-2049</t>
         </is>
       </c>
       <c r="G7" s="5" t="inlineStr">
         <is>
-          <t>SAE J2395
-SAE J1005
-ISO 2575</t>
+          <t>ISO 2575:2021 Cl. 5.2: minimum symbol height 5 mm at design eye point. SAE J1005: symbol ≥3.2 mm; text/numerals ≥4.8 mm. FMVSS 101 S5.3: legible at 76 cm viewing distance.</t>
         </is>
       </c>
       <c r="H7" s="5" t="inlineStr">
@@ -1228,27 +1926,27 @@
       </c>
       <c r="I7" s="5" t="inlineStr">
         <is>
-          <t>Filled-in symbol with text "OFF" beneath the vehicle outline.</t>
+          <t>Filled symbol: headlamp lens with rays pointing rearward through horizontal lines; distinguishable from front fog by rearward ray direction.</t>
         </is>
       </c>
       <c r="J7" s="5" t="inlineStr">
         <is>
-          <t>SAE J387 – minimum luminance of 2.0 cd/m²; maximum of 100 cd/m² to prevent glare at night</t>
+          <t>SAE J387 / ECE R121 Annex 4: minimum luminance 2 cd/m² (night), max 100 cd/m² (to prevent glare). Daytime: 100–1 000 cd/m².</t>
         </is>
       </c>
       <c r="K7" s="5" t="inlineStr">
         <is>
-          <t>SAE J2402 – at least 3:1 for daytime and 4.5:1 or higher for nighttime</t>
+          <t>SAE J2402: ≥3:1 luminance contrast during day; ≥4.5:1 during night. Symbol-to-background ratio.</t>
         </is>
       </c>
       <c r="L7" s="5" t="inlineStr">
         <is>
-          <t>Within the driver's primary field of view</t>
+          <t>Within the driver's primary field of view (FMVSS 101 S5.1). Visible without head movement. Not obscured by steering wheel.</t>
         </is>
       </c>
       <c r="M7" s="5" t="inlineStr">
         <is>
-          <t>Telltale illuminates when the ESC system is manually turned off by the driver (via a switch). It must remain illuminated as long as the system is off.</t>
+          <t>Illuminates when rear fog lamp is activated. Must extinguish automatically when rear fogs are deactivated. Requires deliberate manual activation/deactivation by the driver to prevent unnecessary use in clear conditions.</t>
         </is>
       </c>
       <c r="N7" s="5" t="inlineStr"/>
@@ -1257,61 +1955,61 @@
       <c r="A8" s="2" t="inlineStr"/>
       <c r="B8" s="3" t="inlineStr">
         <is>
-          <t>ESC Active</t>
+          <t>Trailer Direction Indicator</t>
         </is>
       </c>
       <c r="C8" s="3" t="inlineStr">
         <is>
-          <t>Direct – FMVSS 101
-Indirect – FMVSS 108 &amp; 136</t>
+          <t>Direct – FMVSS 101, Table 1, Item 2
+Indirect – FMVSS 108 (49 CFR 571.108)</t>
         </is>
       </c>
       <c r="D8" s="3" t="inlineStr">
         <is>
-          <t>R140</t>
+          <t>UN R48, Annex 5
+UN R55 (coupling devices)
+UN R121</t>
         </is>
       </c>
       <c r="E8" s="3" t="inlineStr"/>
       <c r="F8" s="3" t="inlineStr">
         <is>
-          <t>ISO 7000-0801</t>
+          <t>ISO 2575:2021, Symbol 7000-0258</t>
         </is>
       </c>
       <c r="G8" s="3" t="inlineStr">
         <is>
-          <t>SAE J2395
-SAE J1005
-ISO 2575</t>
+          <t>ISO 2575:2021 Cl. 5.2: minimum symbol height 5 mm at design eye point. SAE J1005: symbol ≥3.2 mm; text/numerals ≥4.8 mm. FMVSS 101 S5.3: legible at 76 cm viewing distance.</t>
         </is>
       </c>
       <c r="H8" s="3" t="inlineStr">
         <is>
-          <t>Amber</t>
+          <t>Green</t>
         </is>
       </c>
       <c r="I8" s="3" t="inlineStr">
         <is>
-          <t>Filled-in vehicle silhouette with skid marks; no text.</t>
+          <t>Arrow symbol supplemented with trailer representation. Distinguishable from standard turn signal telltale. Must flash in sync with trailer turn signals.</t>
         </is>
       </c>
       <c r="J8" s="3" t="inlineStr">
         <is>
-          <t>SAE J387 – minimum luminance of 2.0 cd/m²; maximum of 100 cd/m² to prevent glare at night</t>
+          <t>SAE J387 / ECE R121 Annex 4: minimum luminance 2 cd/m² (night), max 100 cd/m² (to prevent glare). Daytime: 100–1 000 cd/m².</t>
         </is>
       </c>
       <c r="K8" s="3" t="inlineStr">
         <is>
-          <t>SAE J2402 – at least 3:1 for daytime and 4.5:1 or higher for nighttime</t>
+          <t>SAE J2402: ≥3:1 luminance contrast during day; ≥4.5:1 during night. Symbol-to-background ratio.</t>
         </is>
       </c>
       <c r="L8" s="3" t="inlineStr">
         <is>
-          <t>Within the driver's primary field of view</t>
+          <t>Within the driver's primary field of view (FMVSS 101 S5.1). Visible without head movement. Not obscured by steering wheel.</t>
         </is>
       </c>
       <c r="M8" s="3" t="inlineStr">
         <is>
-          <t>Telltale illuminates (flashes) when the ESC system is actively intervening (applying brake force or reducing engine torque to maintain stability).</t>
+          <t>Flashes when the trailer's turn or hazard indicators are active. If a trailer lamp fails, flash rate may differ from the towing vehicle's rate. Only illuminates when a trailer is electrically connected.</t>
         </is>
       </c>
       <c r="N8" s="3" t="inlineStr"/>
@@ -1320,63 +2018,65 @@
       <c r="A9" s="4" t="inlineStr"/>
       <c r="B9" s="5" t="inlineStr">
         <is>
-          <t>ABS</t>
+          <t>Brake System Warning</t>
         </is>
       </c>
       <c r="C9" s="5" t="inlineStr">
         <is>
-          <t>Direct – FMVSS 101
-Indirect – FMVSS 108 &amp; 135</t>
+          <t>Direct – FMVSS 101, Table 1, Item 3
+Indirect – FMVSS 105 (hydraulic brakes), FMVSS 135 (light vehicle brakes)
+(49 CFR 571.105; 571.135)</t>
         </is>
       </c>
       <c r="D9" s="5" t="inlineStr">
         <is>
-          <t>R13H / R139</t>
-        </is>
-      </c>
-      <c r="E9" s="5" t="inlineStr"/>
+          <t>UN R13H (passenger cars, braking)
+UN R121, Table 1</t>
+        </is>
+      </c>
+      <c r="E9" s="5" t="inlineStr">
+        <is>
+          <t>ECE R13H</t>
+        </is>
+      </c>
       <c r="F9" s="5" t="inlineStr">
         <is>
-          <t>ISO 7000-0659</t>
+          <t>ISO 2575:2021, Symbol 7000-0238</t>
         </is>
       </c>
       <c r="G9" s="5" t="inlineStr">
         <is>
-          <t>SAE J2395
-SAE J1005
-ISO 2575</t>
+          <t>ISO 2575:2021 Cl. 5.2: minimum symbol height 5 mm at design eye point. SAE J1005: symbol ≥3.2 mm; text/numerals ≥4.8 mm. FMVSS 101 S5.3: legible at 76 cm viewing distance.</t>
         </is>
       </c>
       <c r="H9" s="5" t="inlineStr">
         <is>
-          <t>Amber</t>
+          <t>Red</t>
         </is>
       </c>
       <c r="I9" s="5" t="inlineStr">
         <is>
-          <t>Filled in. Letters "ABS" displayed inside a circle.</t>
+          <t>Filled symbol: circle with exclamation mark inside, or text 'BRAKE'. Per FMVSS 101, the identifier must include the word BRAKE or the symbol. May not share the Common Display Area with the ESC malfunction, airbag, TPMS, high beam, seat belt, or passenger airbag off telltales (FMVSS 101 S5.2(b)).</t>
         </is>
       </c>
       <c r="J9" s="5" t="inlineStr">
         <is>
-          <t>SAE J387 – minimum luminance of 2.0 cd/m²; maximum of 100 cd/m² to prevent glare at night</t>
+          <t>SAE J387 / ECE R121 Annex 4: minimum luminance 2 cd/m² (night), max 100 cd/m² (to prevent glare). Daytime: 100–1 000 cd/m².</t>
         </is>
       </c>
       <c r="K9" s="5" t="inlineStr">
         <is>
-          <t>SAE J2402 – at least 3:1 for daytime and 4.5:1 or higher for nighttime</t>
+          <t>SAE J2402: ≥3:1 luminance contrast during day; ≥4.5:1 during night. Symbol-to-background ratio.</t>
         </is>
       </c>
       <c r="L9" s="5" t="inlineStr">
         <is>
-          <t>Within the driver's primary field of view</t>
+          <t>Within the driver's primary field of view (FMVSS 101 S5.1). Visible without head movement. Not obscured by steering wheel.</t>
         </is>
       </c>
       <c r="M9" s="5" t="inlineStr">
         <is>
-          <t>Illuminates briefly during the ignition cycle as part of the system self-check.
-It must remain illuminated if the system detects a fault in the anti-lock braking system.
-No flashing state.</t>
+          <t>Illuminates (steady) when: (1) parking brake is applied (FMVSS 105 S5.3.2); (2) hydraulic brake fluid falls below minimum reservoir level; (3) a brake system failure is detected. Mandatory ignition self-check (lamp on at key-on, extinguishes when system OK). No flashing required; steady illumination for all fault conditions.</t>
         </is>
       </c>
       <c r="N9" s="5" t="inlineStr"/>
@@ -1385,31 +2085,34 @@
       <c r="A10" s="2" t="inlineStr"/>
       <c r="B10" s="3" t="inlineStr">
         <is>
-          <t>Seatbelt</t>
+          <t>Parking Brake Applied</t>
         </is>
       </c>
       <c r="C10" s="3" t="inlineStr">
         <is>
-          <t>Direct – FMVSS 101
-Indirect – FMVSS 208</t>
+          <t>Direct – FMVSS 101, Table 1
+Indirect – FMVSS 135 (49 CFR 571.135)</t>
         </is>
       </c>
       <c r="D10" s="3" t="inlineStr">
         <is>
-          <t>R16</t>
-        </is>
-      </c>
-      <c r="E10" s="3" t="inlineStr"/>
+          <t>UN R13H, Annex 7
+UN R121, Table 1</t>
+        </is>
+      </c>
+      <c r="E10" s="3" t="inlineStr">
+        <is>
+          <t>ECE R13H</t>
+        </is>
+      </c>
       <c r="F10" s="3" t="inlineStr">
         <is>
-          <t>ISO 7000-1431</t>
+          <t>ISO 2575:2021, Symbol 7000-0238 (or separate P-symbol)</t>
         </is>
       </c>
       <c r="G10" s="3" t="inlineStr">
         <is>
-          <t>SAE J2395
-SAE J1005
-ISO 2575</t>
+          <t>ISO 2575:2021 Cl. 5.2: minimum symbol height 5 mm at design eye point. SAE J1005: symbol ≥3.2 mm; text/numerals ≥4.8 mm. FMVSS 101 S5.3: legible at 76 cm viewing distance.</t>
         </is>
       </c>
       <c r="H10" s="3" t="inlineStr">
@@ -1419,28 +2122,27 @@
       </c>
       <c r="I10" s="3" t="inlineStr">
         <is>
-          <t>Filled in. Vehicles may include accompanying text such as "SEATBELT" or "FASTEN SEATBELT".</t>
+          <t>Filled circle with letter 'P' or (P) symbol. Some vehicles combine with brake system warning; however, ISO 2575 recommends a separate symbol where feasible.</t>
         </is>
       </c>
       <c r="J10" s="3" t="inlineStr">
         <is>
-          <t>SAE J387 – minimum luminance of 2.0 cd/m²; maximum of 100 cd/m² to prevent glare at night</t>
+          <t>SAE J387 / ECE R121 Annex 4: minimum luminance 2 cd/m² (night), max 100 cd/m² (to prevent glare). Daytime: 100–1 000 cd/m².</t>
         </is>
       </c>
       <c r="K10" s="3" t="inlineStr">
         <is>
-          <t>SAE J2402 – at least 3:1 for daytime and 4.5:1 or higher for nighttime</t>
+          <t>SAE J2402: ≥3:1 luminance contrast during day; ≥4.5:1 during night. Symbol-to-background ratio.</t>
         </is>
       </c>
       <c r="L10" s="3" t="inlineStr">
         <is>
-          <t>Within the driver's primary field of view</t>
+          <t>Within the driver's primary field of view (FMVSS 101 S5.1). Visible without head movement. Not obscured by steering wheel.</t>
         </is>
       </c>
       <c r="M10" s="3" t="inlineStr">
         <is>
-          <t>The telltale illuminates when the ignition is turned on if the driver (or passenger, if applicable) has not fastened their seatbelt.
-It remains illuminated until the seatbelt(s) are securely fastened.</t>
+          <t>Illuminates when parking brake is engaged. Must extinguish immediately when parking brake is fully released. On vehicles with electronic parking brake (EPB), may remain on while EPB is applying or releasing. Driver must be able to notice it before moving the vehicle.</t>
         </is>
       </c>
       <c r="N10" s="3" t="inlineStr"/>
@@ -1449,65 +2151,65 @@
       <c r="A11" s="4" t="inlineStr"/>
       <c r="B11" s="5" t="inlineStr">
         <is>
-          <t>Airbag</t>
+          <t>ABS Malfunction</t>
         </is>
       </c>
       <c r="C11" s="5" t="inlineStr">
         <is>
-          <t>Direct – FMVSS 101
-Indirect – FMVSS 208</t>
-        </is>
-      </c>
-      <c r="D11" s="5" t="inlineStr"/>
+          <t>Direct – FMVSS 101, Table 1
+Indirect – FMVSS 105, FMVSS 135 (49 CFR 571.105/135)</t>
+        </is>
+      </c>
+      <c r="D11" s="5" t="inlineStr">
+        <is>
+          <t>UN R13H, Annex 6
+UN R139 (braking assistance)
+UN R121, Table 1</t>
+        </is>
+      </c>
       <c r="E11" s="5" t="inlineStr">
         <is>
-          <t>ECE 121</t>
+          <t>ECE R13H</t>
         </is>
       </c>
       <c r="F11" s="5" t="inlineStr">
         <is>
-          <t>ISO 7000-0275</t>
+          <t>ISO 2575:2021, Symbol 7000-0659</t>
         </is>
       </c>
       <c r="G11" s="5" t="inlineStr">
         <is>
-          <t>SAE J2395
-SAE J1005
-ISO 2575</t>
+          <t>ISO 2575:2021 Cl. 5.2: minimum symbol height 5 mm at design eye point. SAE J1005: symbol ≥3.2 mm; text/numerals ≥4.8 mm. FMVSS 101 S5.3: legible at 76 cm viewing distance.</t>
         </is>
       </c>
       <c r="H11" s="5" t="inlineStr">
         <is>
-          <t>Amber or Red based on state</t>
+          <t>Amber</t>
         </is>
       </c>
       <c r="I11" s="5" t="inlineStr">
         <is>
-          <t>Filled in. May also include text such as "AIRBAG", "SRS" (Supplemental Restraint System), or "AIRBAG OFF" when indicating deactivation.</t>
+          <t>Filled circle with letters 'ABS' inside. Letters must be legible at the design viewing distance per FMVSS 101 S5.3.</t>
         </is>
       </c>
       <c r="J11" s="5" t="inlineStr">
         <is>
-          <t>SAE J387 – minimum luminance of 2.0 cd/m²; maximum of 100 cd/m² to prevent glare at night</t>
+          <t>SAE J387 / ECE R121 Annex 4: minimum luminance 2 cd/m² (night), max 100 cd/m² (to prevent glare). Daytime: 100–1 000 cd/m².</t>
         </is>
       </c>
       <c r="K11" s="5" t="inlineStr">
         <is>
-          <t>SAE J2402 – at least 3:1 for daytime and 4.5:1 or higher for nighttime</t>
+          <t>SAE J2402: ≥3:1 luminance contrast during day; ≥4.5:1 during night. Symbol-to-background ratio.</t>
         </is>
       </c>
       <c r="L11" s="5" t="inlineStr">
         <is>
-          <t>Within the driver's primary field of view</t>
+          <t>Within the driver's primary field of view (FMVSS 101 S5.1). Visible without head movement. Not obscured by steering wheel.</t>
         </is>
       </c>
       <c r="M11" s="5" t="inlineStr">
         <is>
-          <t>The airbag telltale must illuminate in amber to indicate a malfunction or deactivation.
-In some vehicles, a red telltale may be used in urgent cases (e.g., critical fault).
-Must illuminate during the ignition cycle as part of a system self-check; turns off shortly after the check if the system is functioning properly.
-Must illuminate if there is a fault in the airbag system: malfunction in the airbag deployment system, deactivation of the passenger airbag (e.g., due to child seat detection).
-If the airbag system is disabled, the telltale must clearly indicate the deactivation status (e.g., "Passenger Airbag Off").</t>
+          <t>Illuminates briefly at ignition-on (self-test) then extinguishes if system is healthy. Remains on (steady) if ABS controller detects a malfunction. Normal braking is unaffected; ABS simply deactivates. No flashing state specified. Extinguishes when fault is cleared.</t>
         </is>
       </c>
       <c r="N11" s="5" t="inlineStr"/>
@@ -1516,63 +2218,60 @@
       <c r="A12" s="2" t="inlineStr"/>
       <c r="B12" s="3" t="inlineStr">
         <is>
-          <t>Front Fog</t>
+          <t>ESC Off</t>
         </is>
       </c>
       <c r="C12" s="3" t="inlineStr">
         <is>
-          <t>Direct – FMVSS 101
-Indirect – FMVSS 108</t>
+          <t>Direct – FMVSS 101, Table 1
+Indirect – FMVSS 126 (49 CFR 571.126), FMVSS 136</t>
         </is>
       </c>
       <c r="D12" s="3" t="inlineStr">
         <is>
-          <t>R48</t>
+          <t>UN R140 (electronic stability control)
+UN R121, Table 1</t>
         </is>
       </c>
       <c r="E12" s="3" t="inlineStr"/>
       <c r="F12" s="3" t="inlineStr">
         <is>
-          <t>ISO 7000-2048</t>
+          <t>ISO 2575:2021, Symbol 7000-0801 (with 'OFF' text)</t>
         </is>
       </c>
       <c r="G12" s="3" t="inlineStr">
         <is>
-          <t>SAE J2395
-SAE J1005
-ISO 2575</t>
+          <t>ISO 2575:2021 Cl. 5.2: minimum symbol height 5 mm at design eye point. SAE J1005: symbol ≥3.2 mm; text/numerals ≥4.8 mm. FMVSS 101 S5.3: legible at 76 cm viewing distance.</t>
         </is>
       </c>
       <c r="H12" s="3" t="inlineStr">
         <is>
-          <t>Green</t>
+          <t>Amber</t>
         </is>
       </c>
       <c r="I12" s="3" t="inlineStr">
         <is>
-          <t>Filled in.</t>
+          <t>Filled vehicle silhouette with skid marks and text 'OFF' below symbol. Text 'OFF' required per FMVSS 126 S5.3.1.</t>
         </is>
       </c>
       <c r="J12" s="3" t="inlineStr">
         <is>
-          <t>SAE J387 – minimum luminance of 2.0 cd/m²; maximum of 100 cd/m² to prevent glare at night</t>
+          <t>SAE J387 / ECE R121 Annex 4: minimum luminance 2 cd/m² (night), max 100 cd/m² (to prevent glare). Daytime: 100–1 000 cd/m².</t>
         </is>
       </c>
       <c r="K12" s="3" t="inlineStr">
         <is>
-          <t>SAE J2402 – at least 3:1 for daytime and 4.5:1 or higher for nighttime</t>
+          <t>SAE J2402: ≥3:1 luminance contrast during day; ≥4.5:1 during night. Symbol-to-background ratio.</t>
         </is>
       </c>
       <c r="L12" s="3" t="inlineStr">
         <is>
-          <t>Within the driver's primary field of view</t>
+          <t>Within the driver's primary field of view (FMVSS 101 S5.1). Visible without head movement. Not obscured by steering wheel.</t>
         </is>
       </c>
       <c r="M12" s="3" t="inlineStr">
         <is>
-          <t>The telltale illuminates whenever the front fog lamps are turned on.
-It must turn off automatically when the fog lamps are switched off.
-In vehicles with integrated lighting controls, the front fog lamps (and their telltale) may deactivate automatically when the high beams are engaged.</t>
+          <t>Illuminates (steady) when ESC has been manually deactivated by the driver. Must remain on for entire duration ESC is off. Must re-arm automatically at each new ignition cycle (FMVSS 126 S5.3.2). Extinguishes when ESC is re-enabled.</t>
         </is>
       </c>
       <c r="N12" s="3" t="inlineStr"/>
@@ -1581,31 +2280,30 @@
       <c r="A13" s="4" t="inlineStr"/>
       <c r="B13" s="5" t="inlineStr">
         <is>
-          <t>Rear Fog</t>
+          <t>ESC Active / Malfunction</t>
         </is>
       </c>
       <c r="C13" s="5" t="inlineStr">
         <is>
-          <t>Direct – FMVSS 101
-Indirect – FMVSS 108</t>
+          <t>Direct – FMVSS 101, Table 1
+Indirect – FMVSS 126 (49 CFR 571.126), FMVSS 136</t>
         </is>
       </c>
       <c r="D13" s="5" t="inlineStr">
         <is>
-          <t>R48</t>
+          <t>UN R140 (electronic stability control)
+UN R121, Table 1</t>
         </is>
       </c>
       <c r="E13" s="5" t="inlineStr"/>
       <c r="F13" s="5" t="inlineStr">
         <is>
-          <t>ISO 7000-2049</t>
+          <t>ISO 2575:2021, Symbol 7000-0801</t>
         </is>
       </c>
       <c r="G13" s="5" t="inlineStr">
         <is>
-          <t>SAE J2395
-SAE J1005
-ISO 2575</t>
+          <t>ISO 2575:2021 Cl. 5.2: minimum symbol height 5 mm at design eye point. SAE J1005: symbol ≥3.2 mm; text/numerals ≥4.8 mm. FMVSS 101 S5.3: legible at 76 cm viewing distance.</t>
         </is>
       </c>
       <c r="H13" s="5" t="inlineStr">
@@ -1615,43 +2313,1836 @@
       </c>
       <c r="I13" s="5" t="inlineStr">
         <is>
-          <t>Filled in.</t>
+          <t>Filled vehicle silhouette with skid/tyre marks. No additional text when showing active intervention. Must be distinguishable from ESC Off telltale.</t>
         </is>
       </c>
       <c r="J13" s="5" t="inlineStr">
         <is>
-          <t>SAE J387 – minimum luminance of 2.0 cd/m²; maximum of 100 cd/m² to prevent glare at night</t>
+          <t>SAE J387 / ECE R121 Annex 4: minimum luminance 2 cd/m² (night), max 100 cd/m² (to prevent glare). Daytime: 100–1 000 cd/m².</t>
         </is>
       </c>
       <c r="K13" s="5" t="inlineStr">
         <is>
-          <t>SAE J2402 – at least 3:1 for daytime and 4.5:1 or higher for nighttime</t>
+          <t>SAE J2402: ≥3:1 luminance contrast during day; ≥4.5:1 during night. Symbol-to-background ratio.</t>
         </is>
       </c>
       <c r="L13" s="5" t="inlineStr">
         <is>
-          <t>Within the driver's primary field of view</t>
+          <t>Within the driver's primary field of view (FMVSS 101 S5.1). Visible without head movement. Not obscured by steering wheel.</t>
         </is>
       </c>
       <c r="M13" s="5" t="inlineStr">
         <is>
-          <t>The telltale illuminates whenever the rear fog lamps are turned on.
-It must turn off automatically when the rear fog lamps are deactivated (Manual Deactivation).
-In vehicles with automatic lighting systems, the rear fog lamps (and their telltale) should require manual activation and deactivation by the driver to prevent unnecessary use.</t>
+          <t>FLASHING: ESC is actively intervening (applying selective braking or throttle reduction) to maintain stability. STEADY: ESC system malfunction detected. Must illuminate (steady) within 10 s of fault detection. Extinguishes when fault is cleared.</t>
         </is>
       </c>
       <c r="N13" s="5" t="inlineStr"/>
     </row>
-    <row r="15" ht="18" customHeight="1">
-      <c r="A15" s="6" t="inlineStr">
-        <is>
-          <t>Color key: 🔴 Red = immediate safety hazard  🟡 Amber = driver attention/service required  🟢 Green = normal operational status  🔵 Blue = high-beam headlamp active</t>
+    <row r="14" ht="100" customHeight="1">
+      <c r="A14" s="2" t="inlineStr"/>
+      <c r="B14" s="3" t="inlineStr">
+        <is>
+          <t>Electronic Parking Brake (EPB)</t>
+        </is>
+      </c>
+      <c r="C14" s="3" t="inlineStr">
+        <is>
+          <t>Direct – FMVSS 101, Table 1
+Indirect – FMVSS 135 (49 CFR 571.135)</t>
+        </is>
+      </c>
+      <c r="D14" s="3" t="inlineStr">
+        <is>
+          <t>UN R13H
+UN R121, Table 1</t>
+        </is>
+      </c>
+      <c r="E14" s="3" t="inlineStr">
+        <is>
+          <t>ECE R13H</t>
+        </is>
+      </c>
+      <c r="F14" s="3" t="inlineStr">
+        <is>
+          <t>ISO 2575:2021, Symbol 7000-2060</t>
+        </is>
+      </c>
+      <c r="G14" s="3" t="inlineStr">
+        <is>
+          <t>ISO 2575:2021 Cl. 5.2: minimum symbol height 5 mm at design eye point. SAE J1005: symbol ≥3.2 mm; text/numerals ≥4.8 mm. FMVSS 101 S5.3: legible at 76 cm viewing distance.</t>
+        </is>
+      </c>
+      <c r="H14" s="3" t="inlineStr">
+        <is>
+          <t>Red</t>
+        </is>
+      </c>
+      <c r="I14" s="3" t="inlineStr">
+        <is>
+          <t>Letters 'EPB' inside circle, or filled brake symbol with electric indicator. Must be visually distinct from the manual parking brake telltale where both exist.</t>
+        </is>
+      </c>
+      <c r="J14" s="3" t="inlineStr">
+        <is>
+          <t>SAE J387 / ECE R121 Annex 4: minimum luminance 2 cd/m² (night), max 100 cd/m² (to prevent glare). Daytime: 100–1 000 cd/m².</t>
+        </is>
+      </c>
+      <c r="K14" s="3" t="inlineStr">
+        <is>
+          <t>SAE J2402: ≥3:1 luminance contrast during day; ≥4.5:1 during night. Symbol-to-background ratio.</t>
+        </is>
+      </c>
+      <c r="L14" s="3" t="inlineStr">
+        <is>
+          <t>Within the driver's primary field of view (FMVSS 101 S5.1). Visible without head movement. Not obscured by steering wheel.</t>
+        </is>
+      </c>
+      <c r="M14" s="3" t="inlineStr">
+        <is>
+          <t>Illuminates (steady) when the electronic parking brake is applied. Flashes or shows 'AUTO HOLD' variant during automatic hold function depending on OEM design. Extinguishes when brake is released. A separate amber telltale may indicate EPB system fault.</t>
+        </is>
+      </c>
+      <c r="N14" s="3" t="inlineStr"/>
+    </row>
+    <row r="15" ht="100" customHeight="1">
+      <c r="A15" s="4" t="inlineStr"/>
+      <c r="B15" s="5" t="inlineStr">
+        <is>
+          <t>Tire Pressure Monitoring System (TPMS)</t>
+        </is>
+      </c>
+      <c r="C15" s="5" t="inlineStr">
+        <is>
+          <t>Direct – FMVSS 101, Table 1
+Indirect – FMVSS 138 (49 CFR 571.138)</t>
+        </is>
+      </c>
+      <c r="D15" s="5" t="inlineStr">
+        <is>
+          <t>UN R141 (tyre pressure monitoring)
+UN R121, Table 1</t>
+        </is>
+      </c>
+      <c r="E15" s="5" t="inlineStr"/>
+      <c r="F15" s="5" t="inlineStr">
+        <is>
+          <t>ISO 2575:2021, Symbol 7000-1109</t>
+        </is>
+      </c>
+      <c r="G15" s="5" t="inlineStr">
+        <is>
+          <t>ISO 2575:2021 Cl. 5.2: minimum symbol height 5 mm at design eye point. SAE J1005: symbol ≥3.2 mm; text/numerals ≥4.8 mm. FMVSS 101 S5.3: legible at 76 cm viewing distance.</t>
+        </is>
+      </c>
+      <c r="H15" s="5" t="inlineStr">
+        <is>
+          <t>Amber</t>
+        </is>
+      </c>
+      <c r="I15" s="5" t="inlineStr">
+        <is>
+          <t>Filled symbol: cross-section of tyre with exclamation mark inside. Must be filled, not outline only (FMVSS 138 S5).</t>
+        </is>
+      </c>
+      <c r="J15" s="5" t="inlineStr">
+        <is>
+          <t>SAE J387 / ECE R121 Annex 4: minimum luminance 2 cd/m² (night), max 100 cd/m² (to prevent glare). Daytime: 100–1 000 cd/m².</t>
+        </is>
+      </c>
+      <c r="K15" s="5" t="inlineStr">
+        <is>
+          <t>SAE J2402: ≥3:1 luminance contrast during day; ≥4.5:1 during night. Symbol-to-background ratio.</t>
+        </is>
+      </c>
+      <c r="L15" s="5" t="inlineStr">
+        <is>
+          <t>Within the driver's primary field of view (FMVSS 101 S5.1). Visible without head movement. Not obscured by steering wheel.</t>
+        </is>
+      </c>
+      <c r="M15" s="5" t="inlineStr">
+        <is>
+          <t>STEADY: one or more tyres are significantly under-inflated (FMVSS 138 trigger threshold: ≥25 % below recommended cold inflation pressure). Must illuminate within 10 min of trigger condition. FLASHING (60–90 s then steady): TPMS system malfunction (lost sensor, receiver fault). Must illuminate at each ignition cycle if fault persists.</t>
+        </is>
+      </c>
+      <c r="N15" s="5" t="inlineStr"/>
+    </row>
+    <row r="16" ht="100" customHeight="1">
+      <c r="A16" s="2" t="inlineStr"/>
+      <c r="B16" s="3" t="inlineStr">
+        <is>
+          <t>Low Air Pressure (Pneumatic Brakes)</t>
+        </is>
+      </c>
+      <c r="C16" s="3" t="inlineStr">
+        <is>
+          <t>Direct – FMVSS 101, Table 1
+Indirect – FMVSS 121 (49 CFR 571.121) – Air Brake Systems</t>
+        </is>
+      </c>
+      <c r="D16" s="3" t="inlineStr">
+        <is>
+          <t>UN R13 (braking of heavy vehicles)
+UN R121</t>
+        </is>
+      </c>
+      <c r="E16" s="3" t="inlineStr">
+        <is>
+          <t>ECE R13</t>
+        </is>
+      </c>
+      <c r="F16" s="3" t="inlineStr">
+        <is>
+          <t>ISO 2575:2021, Symbol 7000-0237</t>
+        </is>
+      </c>
+      <c r="G16" s="3" t="inlineStr">
+        <is>
+          <t>ISO 2575:2021 Cl. 5.2: minimum symbol height 5 mm at design eye point. SAE J1005: symbol ≥3.2 mm; text/numerals ≥4.8 mm. FMVSS 101 S5.3: legible at 76 cm viewing distance.</t>
+        </is>
+      </c>
+      <c r="H16" s="3" t="inlineStr">
+        <is>
+          <t>Red</t>
+        </is>
+      </c>
+      <c r="I16" s="3" t="inlineStr">
+        <is>
+          <t>Filled symbol representing compressed air source with warning indicator. Letters 'AIR' acceptable alternative. Mandatory on vehicles equipped with air brakes.</t>
+        </is>
+      </c>
+      <c r="J16" s="3" t="inlineStr">
+        <is>
+          <t>SAE J387 / ECE R121 Annex 4: minimum luminance 2 cd/m² (night), max 100 cd/m² (to prevent glare). Daytime: 100–1 000 cd/m².</t>
+        </is>
+      </c>
+      <c r="K16" s="3" t="inlineStr">
+        <is>
+          <t>SAE J2402: ≥3:1 luminance contrast during day; ≥4.5:1 during night. Symbol-to-background ratio.</t>
+        </is>
+      </c>
+      <c r="L16" s="3" t="inlineStr">
+        <is>
+          <t>Within the driver's primary field of view (FMVSS 101 S5.1). Visible without head movement. Not obscured by steering wheel.</t>
+        </is>
+      </c>
+      <c r="M16" s="3" t="inlineStr">
+        <is>
+          <t>Illuminates when service reservoir air pressure drops below the minimum safe threshold (typically ≤552 kPa / 80 psi per FMVSS 121 S5.2.2). Must illuminate before pressure falls to the point where stopping ability is impaired. Extinguishes when pressure is restored above the threshold.</t>
+        </is>
+      </c>
+      <c r="N16" s="3" t="inlineStr">
+        <is>
+          <t>Passenger car and light truck applications (pneumatic brakes not used).</t>
+        </is>
+      </c>
+    </row>
+    <row r="17" ht="100" customHeight="1">
+      <c r="A17" s="4" t="inlineStr"/>
+      <c r="B17" s="5" t="inlineStr">
+        <is>
+          <t>Malfunction Indicator Lamp (MIL / Check Engine)</t>
+        </is>
+      </c>
+      <c r="C17" s="5" t="inlineStr">
+        <is>
+          <t>Direct – FMVSS 101, Table 2 (voluntary identification)
+Indirect – 40 CFR Part 86 (EPA OBD-II), SAE J1979 (OBD-II diagnostic services), SAE J1930 (terminology)</t>
+        </is>
+      </c>
+      <c r="D17" s="5" t="inlineStr">
+        <is>
+          <t>UN R83 (emissions, light vehicles)
+UN R121</t>
+        </is>
+      </c>
+      <c r="E17" s="5" t="inlineStr"/>
+      <c r="F17" s="5" t="inlineStr">
+        <is>
+          <t>ISO 2575:2021, Symbol 7000-0653</t>
+        </is>
+      </c>
+      <c r="G17" s="5" t="inlineStr">
+        <is>
+          <t>ISO 2575:2021 Cl. 5.2: minimum symbol height 5 mm at design eye point. SAE J1005: symbol ≥3.2 mm; text/numerals ≥4.8 mm. FMVSS 101 S5.3: legible at 76 cm viewing distance.</t>
+        </is>
+      </c>
+      <c r="H17" s="5" t="inlineStr">
+        <is>
+          <t>Amber</t>
+        </is>
+      </c>
+      <c r="I17" s="5" t="inlineStr">
+        <is>
+          <t>Engine silhouette (outline or filled; OEM discretion). Text 'CHECK ENGINE' or 'SERVICE ENGINE SOON' permitted as alternative (SAE J1930). Symbol must be identifiable as the federally required OBD-II MIL.</t>
+        </is>
+      </c>
+      <c r="J17" s="5" t="inlineStr">
+        <is>
+          <t>SAE J387 / ECE R121 Annex 4: minimum luminance 2 cd/m² (night), max 100 cd/m² (to prevent glare). Daytime: 100–1 000 cd/m².</t>
+        </is>
+      </c>
+      <c r="K17" s="5" t="inlineStr">
+        <is>
+          <t>SAE J2402: ≥3:1 luminance contrast during day; ≥4.5:1 during night. Symbol-to-background ratio.</t>
+        </is>
+      </c>
+      <c r="L17" s="5" t="inlineStr">
+        <is>
+          <t>Within the driver's primary field of view (FMVSS 101 S5.1). Visible without head movement. Not obscured by steering wheel.</t>
+        </is>
+      </c>
+      <c r="M17" s="5" t="inlineStr">
+        <is>
+          <t>Illuminates at key-on for self-test (~2–4 s). STEADY: emission-related fault detected by OBD-II (SAE J1979 mode $03 DTCs stored). FLASHING: active misfire severe enough to cause catalytic converter damage; driver must reduce load immediately (SAE J1979). Must extinguish after three consecutive drive cycles without the fault being detected (EPA / SAE J1979).</t>
+        </is>
+      </c>
+      <c r="N17" s="5" t="inlineStr"/>
+    </row>
+    <row r="18" ht="100" customHeight="1">
+      <c r="A18" s="2" t="inlineStr"/>
+      <c r="B18" s="3" t="inlineStr">
+        <is>
+          <t>Engine Oil Pressure Warning</t>
+        </is>
+      </c>
+      <c r="C18" s="3" t="inlineStr">
+        <is>
+          <t>Direct – FMVSS 101, Table 2 (voluntary)
+Indirect – No direct FMVSS; defined by SAE J378 and OEM specifications</t>
+        </is>
+      </c>
+      <c r="D18" s="3" t="inlineStr">
+        <is>
+          <t>UN R121, Table 1</t>
+        </is>
+      </c>
+      <c r="E18" s="3" t="inlineStr"/>
+      <c r="F18" s="3" t="inlineStr">
+        <is>
+          <t>ISO 2575:2021, Symbol 7000-0178</t>
+        </is>
+      </c>
+      <c r="G18" s="3" t="inlineStr">
+        <is>
+          <t>ISO 2575:2021 Cl. 5.2: minimum symbol height 5 mm at design eye point. SAE J1005: symbol ≥3.2 mm; text/numerals ≥4.8 mm. FMVSS 101 S5.3: legible at 76 cm viewing distance.</t>
+        </is>
+      </c>
+      <c r="H18" s="3" t="inlineStr">
+        <is>
+          <t>Red</t>
+        </is>
+      </c>
+      <c r="I18" s="3" t="inlineStr">
+        <is>
+          <t>Filled symbol: oil can / oilpot silhouette with a drop. Must not be confused with oil level symbol. Red indicates immediate action required.</t>
+        </is>
+      </c>
+      <c r="J18" s="3" t="inlineStr">
+        <is>
+          <t>SAE J387 / ECE R121 Annex 4: minimum luminance 2 cd/m² (night), max 100 cd/m² (to prevent glare). Daytime: 100–1 000 cd/m².</t>
+        </is>
+      </c>
+      <c r="K18" s="3" t="inlineStr">
+        <is>
+          <t>SAE J2402: ≥3:1 luminance contrast during day; ≥4.5:1 during night. Symbol-to-background ratio.</t>
+        </is>
+      </c>
+      <c r="L18" s="3" t="inlineStr">
+        <is>
+          <t>Within the driver's primary field of view (FMVSS 101 S5.1). Visible without head movement. Not obscured by steering wheel.</t>
+        </is>
+      </c>
+      <c r="M18" s="3" t="inlineStr">
+        <is>
+          <t>Illuminates (steady) when engine lubrication oil pressure drops below the OEM-specified minimum safe level (typically ~7–14 kPa at idle). Extinguishes within 5 s of key-on when pressure is adequate. Sustained illumination while driving requires immediate engine shutdown to prevent damage. No flashing state.</t>
+        </is>
+      </c>
+      <c r="N18" s="3" t="inlineStr"/>
+    </row>
+    <row r="19" ht="100" customHeight="1">
+      <c r="A19" s="4" t="inlineStr"/>
+      <c r="B19" s="5" t="inlineStr">
+        <is>
+          <t>Engine Coolant Temperature</t>
+        </is>
+      </c>
+      <c r="C19" s="5" t="inlineStr">
+        <is>
+          <t>Direct – FMVSS 101, Table 2 (voluntary)
+Indirect – SAE J292 (cooling system terminology)</t>
+        </is>
+      </c>
+      <c r="D19" s="5" t="inlineStr">
+        <is>
+          <t>UN R121, Table 1</t>
+        </is>
+      </c>
+      <c r="E19" s="5" t="inlineStr"/>
+      <c r="F19" s="5" t="inlineStr">
+        <is>
+          <t>ISO 2575:2021, Symbol 7000-0245</t>
+        </is>
+      </c>
+      <c r="G19" s="5" t="inlineStr">
+        <is>
+          <t>ISO 2575:2021 Cl. 5.2: minimum symbol height 5 mm at design eye point. SAE J1005: symbol ≥3.2 mm; text/numerals ≥4.8 mm. FMVSS 101 S5.3: legible at 76 cm viewing distance.</t>
+        </is>
+      </c>
+      <c r="H19" s="5" t="inlineStr">
+        <is>
+          <t>Red (high temp) / Blue (low temp, OEM optional)</t>
+        </is>
+      </c>
+      <c r="I19" s="5" t="inlineStr">
+        <is>
+          <t>Thermometer-in-water symbol. Red version = dangerously high temperature. Blue version (where used) = engine not yet at operating temperature. ISO 2575 specifies two variants.</t>
+        </is>
+      </c>
+      <c r="J19" s="5" t="inlineStr">
+        <is>
+          <t>SAE J387 / ECE R121 Annex 4: minimum luminance 2 cd/m² (night), max 100 cd/m² (to prevent glare). Daytime: 100–1 000 cd/m².</t>
+        </is>
+      </c>
+      <c r="K19" s="5" t="inlineStr">
+        <is>
+          <t>SAE J2402: ≥3:1 luminance contrast during day; ≥4.5:1 during night. Symbol-to-background ratio.</t>
+        </is>
+      </c>
+      <c r="L19" s="5" t="inlineStr">
+        <is>
+          <t>Within the driver's primary field of view (FMVSS 101 S5.1). Visible without head movement. Not obscured by steering wheel.</t>
+        </is>
+      </c>
+      <c r="M19" s="5" t="inlineStr">
+        <is>
+          <t>RED (steady): coolant temperature has exceeded the safe maximum (typically ~118–121 °C / ~244–250 °F). Driver must stop and allow engine to cool. Continued operation risks engine damage. Blue variant extinguishes once engine reaches normal operating temperature.</t>
+        </is>
+      </c>
+      <c r="N19" s="5" t="inlineStr"/>
+    </row>
+    <row r="20" ht="100" customHeight="1">
+      <c r="A20" s="2" t="inlineStr"/>
+      <c r="B20" s="3" t="inlineStr">
+        <is>
+          <t>Battery / Charging System</t>
+        </is>
+      </c>
+      <c r="C20" s="3" t="inlineStr">
+        <is>
+          <t>Direct – FMVSS 101, Table 2 (voluntary)
+Indirect – SAE J541 (storage battery classification)</t>
+        </is>
+      </c>
+      <c r="D20" s="3" t="inlineStr">
+        <is>
+          <t>UN R121, Table 1</t>
+        </is>
+      </c>
+      <c r="E20" s="3" t="inlineStr"/>
+      <c r="F20" s="3" t="inlineStr">
+        <is>
+          <t>ISO 2575:2021, Symbol 7000-0064</t>
+        </is>
+      </c>
+      <c r="G20" s="3" t="inlineStr">
+        <is>
+          <t>ISO 2575:2021 Cl. 5.2: minimum symbol height 5 mm at design eye point. SAE J1005: symbol ≥3.2 mm; text/numerals ≥4.8 mm. FMVSS 101 S5.3: legible at 76 cm viewing distance.</t>
+        </is>
+      </c>
+      <c r="H20" s="3" t="inlineStr">
+        <is>
+          <t>Red</t>
+        </is>
+      </c>
+      <c r="I20" s="3" t="inlineStr">
+        <is>
+          <t>Battery symbol (rectangle with + and − terminals and two nubs on top). Must be distinguishable from EV high-voltage battery symbol. Filled or outline acceptable.</t>
+        </is>
+      </c>
+      <c r="J20" s="3" t="inlineStr">
+        <is>
+          <t>SAE J387 / ECE R121 Annex 4: minimum luminance 2 cd/m² (night), max 100 cd/m² (to prevent glare). Daytime: 100–1 000 cd/m².</t>
+        </is>
+      </c>
+      <c r="K20" s="3" t="inlineStr">
+        <is>
+          <t>SAE J2402: ≥3:1 luminance contrast during day; ≥4.5:1 during night. Symbol-to-background ratio.</t>
+        </is>
+      </c>
+      <c r="L20" s="3" t="inlineStr">
+        <is>
+          <t>Within the driver's primary field of view (FMVSS 101 S5.1). Visible without head movement. Not obscured by steering wheel.</t>
+        </is>
+      </c>
+      <c r="M20" s="3" t="inlineStr">
+        <is>
+          <t>Illuminates (steady) when the alternator/generator is not charging the battery (charging system voltage below ~12.5 V DC at normal engine speed) or battery voltage is critically low. Extinguishes once charging is restored. Illuminates briefly at key-on as self-test.</t>
+        </is>
+      </c>
+      <c r="N20" s="3" t="inlineStr"/>
+    </row>
+    <row r="21" ht="100" customHeight="1">
+      <c r="A21" s="4" t="inlineStr"/>
+      <c r="B21" s="5" t="inlineStr">
+        <is>
+          <t>Low Fuel Level</t>
+        </is>
+      </c>
+      <c r="C21" s="5" t="inlineStr">
+        <is>
+          <t>Direct – FMVSS 101, Table 2 (voluntary)
+Indirect – SAE J1297 (fuel systems)</t>
+        </is>
+      </c>
+      <c r="D21" s="5" t="inlineStr">
+        <is>
+          <t>UN R121, Table 1</t>
+        </is>
+      </c>
+      <c r="E21" s="5" t="inlineStr"/>
+      <c r="F21" s="5" t="inlineStr">
+        <is>
+          <t>ISO 2575:2021, Symbol 7000-0007</t>
+        </is>
+      </c>
+      <c r="G21" s="5" t="inlineStr">
+        <is>
+          <t>ISO 2575:2021 Cl. 5.2: minimum symbol height 5 mm at design eye point. SAE J1005: symbol ≥3.2 mm; text/numerals ≥4.8 mm. FMVSS 101 S5.3: legible at 76 cm viewing distance.</t>
+        </is>
+      </c>
+      <c r="H21" s="5" t="inlineStr">
+        <is>
+          <t>Amber</t>
+        </is>
+      </c>
+      <c r="I21" s="5" t="inlineStr">
+        <is>
+          <t>Fuel pump / petrol-pump silhouette symbol. Filled. Some vehicles display remaining range or bar-graph supplement alongside the telltale.</t>
+        </is>
+      </c>
+      <c r="J21" s="5" t="inlineStr">
+        <is>
+          <t>SAE J387 / ECE R121 Annex 4: minimum luminance 2 cd/m² (night), max 100 cd/m² (to prevent glare). Daytime: 100–1 000 cd/m².</t>
+        </is>
+      </c>
+      <c r="K21" s="5" t="inlineStr">
+        <is>
+          <t>SAE J2402: ≥3:1 luminance contrast during day; ≥4.5:1 during night. Symbol-to-background ratio.</t>
+        </is>
+      </c>
+      <c r="L21" s="5" t="inlineStr">
+        <is>
+          <t>Within the driver's primary field of view (FMVSS 101 S5.1). Visible without head movement. Not obscured by steering wheel.</t>
+        </is>
+      </c>
+      <c r="M21" s="5" t="inlineStr">
+        <is>
+          <t>Illuminates when fuel level drops below the OEM-specified low-fuel threshold (typically final ~10–15 % of tank capacity). May flash to indicate critically low level (design-dependent). Extinguishes after refuelling above the threshold.</t>
+        </is>
+      </c>
+      <c r="N21" s="5" t="inlineStr"/>
+    </row>
+    <row r="22" ht="100" customHeight="1">
+      <c r="A22" s="2" t="inlineStr"/>
+      <c r="B22" s="3" t="inlineStr">
+        <is>
+          <t>Glow Plug (Diesel Pre-heat)</t>
+        </is>
+      </c>
+      <c r="C22" s="3" t="inlineStr">
+        <is>
+          <t>Direct – FMVSS 101, Table 2 (voluntary)
+Indirect – EPA 40 CFR Part 86 (diesel emissions)</t>
+        </is>
+      </c>
+      <c r="D22" s="3" t="inlineStr">
+        <is>
+          <t>UN R83 (diesel emissions); UN R121</t>
+        </is>
+      </c>
+      <c r="E22" s="3" t="inlineStr"/>
+      <c r="F22" s="3" t="inlineStr">
+        <is>
+          <t>ISO 2575:2021, Symbol 7000-0273</t>
+        </is>
+      </c>
+      <c r="G22" s="3" t="inlineStr">
+        <is>
+          <t>ISO 2575:2021 Cl. 5.2: minimum symbol height 5 mm at design eye point. SAE J1005: symbol ≥3.2 mm; text/numerals ≥4.8 mm. FMVSS 101 S5.3: legible at 76 cm viewing distance.</t>
+        </is>
+      </c>
+      <c r="H22" s="3" t="inlineStr">
+        <is>
+          <t>Amber</t>
+        </is>
+      </c>
+      <c r="I22" s="3" t="inlineStr">
+        <is>
+          <t>Coiled wire / heater element symbol (glow-plug shape). Filled. Applicable only to diesel and some alternative-fuel engines with pre-heat systems.</t>
+        </is>
+      </c>
+      <c r="J22" s="3" t="inlineStr">
+        <is>
+          <t>SAE J387 / ECE R121 Annex 4: minimum luminance 2 cd/m² (night), max 100 cd/m² (to prevent glare). Daytime: 100–1 000 cd/m².</t>
+        </is>
+      </c>
+      <c r="K22" s="3" t="inlineStr">
+        <is>
+          <t>SAE J2402: ≥3:1 luminance contrast during day; ≥4.5:1 during night. Symbol-to-background ratio.</t>
+        </is>
+      </c>
+      <c r="L22" s="3" t="inlineStr">
+        <is>
+          <t>Within the driver's primary field of view (FMVSS 101 S5.1). Visible without head movement. Not obscured by steering wheel.</t>
+        </is>
+      </c>
+      <c r="M22" s="3" t="inlineStr">
+        <is>
+          <t>Illuminates when glow plugs are being energised prior to engine start in cold conditions. Extinguishes when cylinders are sufficiently warm for reliable ignition. STEADY + long duration: glow plug fault. On some systems, flashing indicates a glow plug circuit malfunction.</t>
+        </is>
+      </c>
+      <c r="N22" s="3" t="inlineStr">
+        <is>
+          <t>Gasoline/petrol engine vehicles without pre-heat systems.</t>
+        </is>
+      </c>
+    </row>
+    <row r="23" ht="100" customHeight="1">
+      <c r="A23" s="4" t="inlineStr"/>
+      <c r="B23" s="5" t="inlineStr">
+        <is>
+          <t>Service / Maintenance Required</t>
+        </is>
+      </c>
+      <c r="C23" s="5" t="inlineStr">
+        <is>
+          <t>Direct – FMVSS 101, Table 2 (voluntary)
+Indirect – OEM service interval algorithm</t>
+        </is>
+      </c>
+      <c r="D23" s="5" t="inlineStr">
+        <is>
+          <t>UN R121, Table 1</t>
+        </is>
+      </c>
+      <c r="E23" s="5" t="inlineStr"/>
+      <c r="F23" s="5" t="inlineStr">
+        <is>
+          <t>ISO 2575:2021, Symbol 7000-0453</t>
+        </is>
+      </c>
+      <c r="G23" s="5" t="inlineStr">
+        <is>
+          <t>ISO 2575:2021 Cl. 5.2: minimum symbol height 5 mm at design eye point. SAE J1005: symbol ≥3.2 mm; text/numerals ≥4.8 mm. FMVSS 101 S5.3: legible at 76 cm viewing distance.</t>
+        </is>
+      </c>
+      <c r="H23" s="5" t="inlineStr">
+        <is>
+          <t>Amber</t>
+        </is>
+      </c>
+      <c r="I23" s="5" t="inlineStr">
+        <is>
+          <t>Wrench / spanner symbol or text 'SERVICE'. Not to be confused with MIL. Some manufacturers use a separate oil change indicator.</t>
+        </is>
+      </c>
+      <c r="J23" s="5" t="inlineStr">
+        <is>
+          <t>SAE J387 / ECE R121 Annex 4: minimum luminance 2 cd/m² (night), max 100 cd/m² (to prevent glare). Daytime: 100–1 000 cd/m².</t>
+        </is>
+      </c>
+      <c r="K23" s="5" t="inlineStr">
+        <is>
+          <t>SAE J2402: ≥3:1 luminance contrast during day; ≥4.5:1 during night. Symbol-to-background ratio.</t>
+        </is>
+      </c>
+      <c r="L23" s="5" t="inlineStr">
+        <is>
+          <t>Within the driver's primary field of view (FMVSS 101 S5.1). Visible without head movement. Not obscured by steering wheel.</t>
+        </is>
+      </c>
+      <c r="M23" s="5" t="inlineStr">
+        <is>
+          <t>Illuminates when the vehicle's service interval monitor (based on mileage, time, or oil quality algorithm) determines scheduled maintenance is due. Extinguishes after dealer reset or manual reset per the owner's manual procedure. Does not indicate an active fault.</t>
+        </is>
+      </c>
+      <c r="N23" s="5" t="inlineStr"/>
+    </row>
+    <row r="24" ht="100" customHeight="1">
+      <c r="A24" s="2" t="inlineStr"/>
+      <c r="B24" s="3" t="inlineStr">
+        <is>
+          <t>Traction Control Active</t>
+        </is>
+      </c>
+      <c r="C24" s="3" t="inlineStr">
+        <is>
+          <t>Direct – FMVSS 101, Table 1 (combined with ESC per FMVSS 126)
+Indirect – FMVSS 126 (49 CFR 571.126)</t>
+        </is>
+      </c>
+      <c r="D24" s="3" t="inlineStr">
+        <is>
+          <t>UN R140 (ESC)
+UN R121, Table 1</t>
+        </is>
+      </c>
+      <c r="E24" s="3" t="inlineStr"/>
+      <c r="F24" s="3" t="inlineStr">
+        <is>
+          <t>ISO 2575:2021, Symbol 7000-0800</t>
+        </is>
+      </c>
+      <c r="G24" s="3" t="inlineStr">
+        <is>
+          <t>ISO 2575:2021 Cl. 5.2: minimum symbol height 5 mm at design eye point. SAE J1005: symbol ≥3.2 mm; text/numerals ≥4.8 mm. FMVSS 101 S5.3: legible at 76 cm viewing distance.</t>
+        </is>
+      </c>
+      <c r="H24" s="3" t="inlineStr">
+        <is>
+          <t>Amber</t>
+        </is>
+      </c>
+      <c r="I24" s="3" t="inlineStr">
+        <is>
+          <t>Vehicle silhouette with tyre-slip marks; similar to ESC symbol but without text 'OFF'. May include 'TC' sub-label. Must be distinguishable from ESC malfunction telltale.</t>
+        </is>
+      </c>
+      <c r="J24" s="3" t="inlineStr">
+        <is>
+          <t>SAE J387 / ECE R121 Annex 4: minimum luminance 2 cd/m² (night), max 100 cd/m² (to prevent glare). Daytime: 100–1 000 cd/m².</t>
+        </is>
+      </c>
+      <c r="K24" s="3" t="inlineStr">
+        <is>
+          <t>SAE J2402: ≥3:1 luminance contrast during day; ≥4.5:1 during night. Symbol-to-background ratio.</t>
+        </is>
+      </c>
+      <c r="L24" s="3" t="inlineStr">
+        <is>
+          <t>Within the driver's primary field of view (FMVSS 101 S5.1). Visible without head movement. Not obscured by steering wheel.</t>
+        </is>
+      </c>
+      <c r="M24" s="3" t="inlineStr">
+        <is>
+          <t>Flashes when traction control is actively limiting wheel spin (reducing engine torque or applying selective braking). Illuminates steady if the traction control system has a malfunction. On vehicles where traction control and ESC share one symbol (FMVSS 126), this telltale serves both functions.</t>
+        </is>
+      </c>
+      <c r="N24" s="3" t="inlineStr"/>
+    </row>
+    <row r="25" ht="100" customHeight="1">
+      <c r="A25" s="4" t="inlineStr"/>
+      <c r="B25" s="5" t="inlineStr">
+        <is>
+          <t>Seat Belt Reminder</t>
+        </is>
+      </c>
+      <c r="C25" s="5" t="inlineStr">
+        <is>
+          <t>Direct – FMVSS 101, Table 1, Item 5
+Indirect – FMVSS 208 (49 CFR 571.208) – Occupant Crash Protection</t>
+        </is>
+      </c>
+      <c r="D25" s="5" t="inlineStr">
+        <is>
+          <t>UN R16 (safety belts)
+UN R121, Table 1</t>
+        </is>
+      </c>
+      <c r="E25" s="5" t="inlineStr"/>
+      <c r="F25" s="5" t="inlineStr">
+        <is>
+          <t>ISO 2575:2021, Symbol 7000-1431</t>
+        </is>
+      </c>
+      <c r="G25" s="5" t="inlineStr">
+        <is>
+          <t>ISO 2575:2021 Cl. 5.2: minimum symbol height 5 mm at design eye point. SAE J1005: symbol ≥3.2 mm; text/numerals ≥4.8 mm. FMVSS 101 S5.3: legible at 76 cm viewing distance.</t>
+        </is>
+      </c>
+      <c r="H25" s="5" t="inlineStr">
+        <is>
+          <t>Red</t>
+        </is>
+      </c>
+      <c r="I25" s="5" t="inlineStr">
+        <is>
+          <t>Filled seated-occupant figure with diagonal seat belt strap. Text 'FASTEN SEAT BELT' or 'SEATBELT' may supplement. FMVSS 208 specifies a separate front and rear occupant reminder for new platforms.</t>
+        </is>
+      </c>
+      <c r="J25" s="5" t="inlineStr">
+        <is>
+          <t>SAE J387 / ECE R121 Annex 4: minimum luminance 2 cd/m² (night), max 100 cd/m² (to prevent glare). Daytime: 100–1 000 cd/m².</t>
+        </is>
+      </c>
+      <c r="K25" s="5" t="inlineStr">
+        <is>
+          <t>SAE J2402: ≥3:1 luminance contrast during day; ≥4.5:1 during night. Symbol-to-background ratio.</t>
+        </is>
+      </c>
+      <c r="L25" s="5" t="inlineStr">
+        <is>
+          <t>Within the driver's primary field of view (FMVSS 101 S5.1). Visible without head movement. Not obscured by steering wheel.</t>
+        </is>
+      </c>
+      <c r="M25" s="5" t="inlineStr">
+        <is>
+          <t>Illuminates at ignition-on if driver (and/or front passenger where equipped) seat belt is not fastened. FMVSS 208 S4.5.3.3: audible/visual reminder sequence must begin within 60 s of engine start. Extinguishes when belt is buckled. Supplemental rear-seat indicators for MY 2026+ (FMVSS 208 amendment).</t>
+        </is>
+      </c>
+      <c r="N25" s="5" t="inlineStr"/>
+    </row>
+    <row r="26" ht="100" customHeight="1">
+      <c r="A26" s="2" t="inlineStr"/>
+      <c r="B26" s="3" t="inlineStr">
+        <is>
+          <t>Supplemental Restraint System / Airbag Malfunction</t>
+        </is>
+      </c>
+      <c r="C26" s="3" t="inlineStr">
+        <is>
+          <t>Direct – FMVSS 101, Table 1
+Indirect – FMVSS 208 (49 CFR 571.208)</t>
+        </is>
+      </c>
+      <c r="D26" s="3" t="inlineStr">
+        <is>
+          <t>UN R94 (frontal collision)
+UN R95 (lateral collision)
+UN R121, Table 1</t>
+        </is>
+      </c>
+      <c r="E26" s="3" t="inlineStr">
+        <is>
+          <t>ECE R121</t>
+        </is>
+      </c>
+      <c r="F26" s="3" t="inlineStr">
+        <is>
+          <t>ISO 2575:2021, Symbol 7000-0275</t>
+        </is>
+      </c>
+      <c r="G26" s="3" t="inlineStr">
+        <is>
+          <t>ISO 2575:2021 Cl. 5.2: minimum symbol height 5 mm at design eye point. SAE J1005: symbol ≥3.2 mm; text/numerals ≥4.8 mm. FMVSS 101 S5.3: legible at 76 cm viewing distance.</t>
+        </is>
+      </c>
+      <c r="H26" s="3" t="inlineStr">
+        <is>
+          <t>Amber (malfunction); Red (critical fault / OEM option)</t>
+        </is>
+      </c>
+      <c r="I26" s="3" t="inlineStr">
+        <is>
+          <t>Filled seated-occupant figure with deploying airbag balloon. Text 'AIRBAG', 'SRS', or 'AIRBAG OFF' for deactivation variant. FMVSS 208 S4.5.4 requires the exact lamp function.</t>
+        </is>
+      </c>
+      <c r="J26" s="3" t="inlineStr">
+        <is>
+          <t>SAE J387 / ECE R121 Annex 4: minimum luminance 2 cd/m² (night), max 100 cd/m² (to prevent glare). Daytime: 100–1 000 cd/m².</t>
+        </is>
+      </c>
+      <c r="K26" s="3" t="inlineStr">
+        <is>
+          <t>SAE J2402: ≥3:1 luminance contrast during day; ≥4.5:1 during night. Symbol-to-background ratio.</t>
+        </is>
+      </c>
+      <c r="L26" s="3" t="inlineStr">
+        <is>
+          <t>Within the driver's primary field of view (FMVSS 101 S5.1). Visible without head movement. Not obscured by steering wheel.</t>
+        </is>
+      </c>
+      <c r="M26" s="3" t="inlineStr">
+        <is>
+          <t>Illuminates at key-on (self-test, ~4–8 s) then extinguishes. STEADY (amber): SRS controller detects fault (e.g., clock spring, sensor, squib circuit). Driver must service system. A red lamp may indicate critical fault requiring immediate attention (OEM). A separate 'PAB OFF' telltale illuminates when passenger airbag is disabled (child seat/OCS sensor).</t>
+        </is>
+      </c>
+      <c r="N26" s="3" t="inlineStr"/>
+    </row>
+    <row r="27" ht="100" customHeight="1">
+      <c r="A27" s="4" t="inlineStr"/>
+      <c r="B27" s="5" t="inlineStr">
+        <is>
+          <t>Passenger Airbag Off</t>
+        </is>
+      </c>
+      <c r="C27" s="5" t="inlineStr">
+        <is>
+          <t>Direct – FMVSS 101, Table 1
+Indirect – FMVSS 208 (49 CFR 571.208) S4.5.4.2</t>
+        </is>
+      </c>
+      <c r="D27" s="5" t="inlineStr">
+        <is>
+          <t>UN R94
+UN R121</t>
+        </is>
+      </c>
+      <c r="E27" s="5" t="inlineStr"/>
+      <c r="F27" s="5" t="inlineStr">
+        <is>
+          <t>ISO 2575:2021, Symbol 7000-2029</t>
+        </is>
+      </c>
+      <c r="G27" s="5" t="inlineStr">
+        <is>
+          <t>ISO 2575:2021 Cl. 5.2: minimum symbol height 5 mm at design eye point. SAE J1005: symbol ≥3.2 mm; text/numerals ≥4.8 mm. FMVSS 101 S5.3: legible at 76 cm viewing distance.</t>
+        </is>
+      </c>
+      <c r="H27" s="5" t="inlineStr">
+        <is>
+          <t>Amber</t>
+        </is>
+      </c>
+      <c r="I27" s="5" t="inlineStr">
+        <is>
+          <t>Airbag symbol with X-slash or text 'PASSENGER AIRBAG OFF'. FMVSS 208 mandates a specific illuminated label visible to both front occupants.</t>
+        </is>
+      </c>
+      <c r="J27" s="5" t="inlineStr">
+        <is>
+          <t>SAE J387 / ECE R121 Annex 4: minimum luminance 2 cd/m² (night), max 100 cd/m² (to prevent glare). Daytime: 100–1 000 cd/m².</t>
+        </is>
+      </c>
+      <c r="K27" s="5" t="inlineStr">
+        <is>
+          <t>SAE J2402: ≥3:1 luminance contrast during day; ≥4.5:1 during night. Symbol-to-background ratio.</t>
+        </is>
+      </c>
+      <c r="L27" s="5" t="inlineStr">
+        <is>
+          <t>Within the driver's primary field of view (FMVSS 101 S5.1). Visible without head movement. Not obscured by steering wheel.</t>
+        </is>
+      </c>
+      <c r="M27" s="5" t="inlineStr">
+        <is>
+          <t>Illuminates (steady) when the passenger frontal airbag is suppressed (due to OCS child-seat detection, manual switch, or key-switch). Must remain on as long as airbag is suppressed. Extinguishes when adult occupant is detected or manual switch is reset. FMVSS 208 S4.5.4.2 requires this telltale to be readable in both day and night.</t>
+        </is>
+      </c>
+      <c r="N27" s="5" t="inlineStr"/>
+    </row>
+    <row r="28" ht="100" customHeight="1">
+      <c r="A28" s="2" t="inlineStr"/>
+      <c r="B28" s="3" t="inlineStr">
+        <is>
+          <t>Door Ajar</t>
+        </is>
+      </c>
+      <c r="C28" s="3" t="inlineStr">
+        <is>
+          <t>Direct – FMVSS 101, Table 2 (voluntary)
+Indirect – FMVSS 206 (door locks and retention)</t>
+        </is>
+      </c>
+      <c r="D28" s="3" t="inlineStr">
+        <is>
+          <t>UN R121, Table 1</t>
+        </is>
+      </c>
+      <c r="E28" s="3" t="inlineStr"/>
+      <c r="F28" s="3" t="inlineStr">
+        <is>
+          <t>ISO 2575:2021, Symbol 7000-0451</t>
+        </is>
+      </c>
+      <c r="G28" s="3" t="inlineStr">
+        <is>
+          <t>ISO 2575:2021 Cl. 5.2: minimum symbol height 5 mm at design eye point. SAE J1005: symbol ≥3.2 mm; text/numerals ≥4.8 mm. FMVSS 101 S5.3: legible at 76 cm viewing distance.</t>
+        </is>
+      </c>
+      <c r="H28" s="3" t="inlineStr">
+        <is>
+          <t>Red (door open) or Amber (ajar / not fully latched)</t>
+        </is>
+      </c>
+      <c r="I28" s="3" t="inlineStr">
+        <is>
+          <t>Top-view vehicle outline with one or more doors shown open/angled outward. Individual door indicators may highlight the specific open door.</t>
+        </is>
+      </c>
+      <c r="J28" s="3" t="inlineStr">
+        <is>
+          <t>SAE J387 / ECE R121 Annex 4: minimum luminance 2 cd/m² (night), max 100 cd/m² (to prevent glare). Daytime: 100–1 000 cd/m².</t>
+        </is>
+      </c>
+      <c r="K28" s="3" t="inlineStr">
+        <is>
+          <t>SAE J2402: ≥3:1 luminance contrast during day; ≥4.5:1 during night. Symbol-to-background ratio.</t>
+        </is>
+      </c>
+      <c r="L28" s="3" t="inlineStr">
+        <is>
+          <t>Within the driver's primary field of view (FMVSS 101 S5.1). Visible without head movement. Not obscured by steering wheel.</t>
+        </is>
+      </c>
+      <c r="M28" s="3" t="inlineStr">
+        <is>
+          <t>Illuminates when any door/boot/bonnet is not fully latched. May show individual icons per door or a single generic indicator. Extinguishes when all doors/hatches are fully closed and latched. At vehicle speeds &gt; ~8 km/h, may activate audible chime in addition to visual.</t>
+        </is>
+      </c>
+      <c r="N28" s="3" t="inlineStr"/>
+    </row>
+    <row r="29" ht="100" customHeight="1">
+      <c r="A29" s="4" t="inlineStr"/>
+      <c r="B29" s="5" t="inlineStr">
+        <is>
+          <t>Washer Fluid Level Low</t>
+        </is>
+      </c>
+      <c r="C29" s="5" t="inlineStr">
+        <is>
+          <t>Direct – FMVSS 101, Table 2 (voluntary)
+Indirect – SAE J942 (windscreen wiper systems)</t>
+        </is>
+      </c>
+      <c r="D29" s="5" t="inlineStr">
+        <is>
+          <t>UN R121, Table 1</t>
+        </is>
+      </c>
+      <c r="E29" s="5" t="inlineStr"/>
+      <c r="F29" s="5" t="inlineStr">
+        <is>
+          <t>ISO 2575:2021, Symbol 7000-0183</t>
+        </is>
+      </c>
+      <c r="G29" s="5" t="inlineStr">
+        <is>
+          <t>ISO 2575:2021 Cl. 5.2: minimum symbol height 5 mm at design eye point. SAE J1005: symbol ≥3.2 mm; text/numerals ≥4.8 mm. FMVSS 101 S5.3: legible at 76 cm viewing distance.</t>
+        </is>
+      </c>
+      <c r="H29" s="5" t="inlineStr">
+        <is>
+          <t>Amber</t>
+        </is>
+      </c>
+      <c r="I29" s="5" t="inlineStr">
+        <is>
+          <t>Windscreen/washer bottle symbol with fluid drops. Filled. Not safety-critical; amber appropriate for 'service soon'.</t>
+        </is>
+      </c>
+      <c r="J29" s="5" t="inlineStr">
+        <is>
+          <t>SAE J387 / ECE R121 Annex 4: minimum luminance 2 cd/m² (night), max 100 cd/m² (to prevent glare). Daytime: 100–1 000 cd/m².</t>
+        </is>
+      </c>
+      <c r="K29" s="5" t="inlineStr">
+        <is>
+          <t>SAE J2402: ≥3:1 luminance contrast during day; ≥4.5:1 during night. Symbol-to-background ratio.</t>
+        </is>
+      </c>
+      <c r="L29" s="5" t="inlineStr">
+        <is>
+          <t>Within the driver's primary field of view (FMVSS 101 S5.1). Visible without head movement. Not obscured by steering wheel.</t>
+        </is>
+      </c>
+      <c r="M29" s="5" t="inlineStr">
+        <is>
+          <t>Illuminates when windshield washer fluid reservoir drops below the minimum level (OEM-defined). Extinguishes when reservoir is refilled above the threshold. Non-critical indicator; no audible chime required.</t>
+        </is>
+      </c>
+      <c r="N29" s="5" t="inlineStr"/>
+    </row>
+    <row r="30" ht="100" customHeight="1">
+      <c r="A30" s="2" t="inlineStr"/>
+      <c r="B30" s="3" t="inlineStr">
+        <is>
+          <t>Immobiliser / Security / Anti-Theft</t>
+        </is>
+      </c>
+      <c r="C30" s="3" t="inlineStr">
+        <is>
+          <t>Direct – FMVSS 101, Table 2 (voluntary)
+Indirect – SAE J2061 (theft deterrent)</t>
+        </is>
+      </c>
+      <c r="D30" s="3" t="inlineStr">
+        <is>
+          <t>UN R116 (protection against unauthorized use)
+UN R121</t>
+        </is>
+      </c>
+      <c r="E30" s="3" t="inlineStr">
+        <is>
+          <t>ECE R116</t>
+        </is>
+      </c>
+      <c r="F30" s="3" t="inlineStr">
+        <is>
+          <t>ISO 2575:2021, Symbol 7000-1534</t>
+        </is>
+      </c>
+      <c r="G30" s="3" t="inlineStr">
+        <is>
+          <t>ISO 2575:2021 Cl. 5.2: minimum symbol height 5 mm at design eye point. SAE J1005: symbol ≥3.2 mm; text/numerals ≥4.8 mm. FMVSS 101 S5.3: legible at 76 cm viewing distance.</t>
+        </is>
+      </c>
+      <c r="H30" s="3" t="inlineStr">
+        <is>
+          <t>Red (armed/fault) or Green (disarmed/OK, OEM-dependent)</t>
+        </is>
+      </c>
+      <c r="I30" s="3" t="inlineStr">
+        <is>
+          <t>Vehicle with padlock or key symbol. Red = security system armed or fault. Green = correctly disarmed. OEM practice varies widely; ISO 2575 specifies the standard symbol.</t>
+        </is>
+      </c>
+      <c r="J30" s="3" t="inlineStr">
+        <is>
+          <t>SAE J387 / ECE R121 Annex 4: minimum luminance 2 cd/m² (night), max 100 cd/m² (to prevent glare). Daytime: 100–1 000 cd/m².</t>
+        </is>
+      </c>
+      <c r="K30" s="3" t="inlineStr">
+        <is>
+          <t>SAE J2402: ≥3:1 luminance contrast during day; ≥4.5:1 during night. Symbol-to-background ratio.</t>
+        </is>
+      </c>
+      <c r="L30" s="3" t="inlineStr">
+        <is>
+          <t>Within the driver's primary field of view (FMVSS 101 S5.1). Visible without head movement. Not obscured by steering wheel.</t>
+        </is>
+      </c>
+      <c r="M30" s="3" t="inlineStr">
+        <is>
+          <t>STEADY RED: immobiliser is active and vehicle will not start, or the ECM/BCM has not received a valid key signal. FLASHING RED: vehicle's alarm system is armed (parked). Extinguishes (or turns green) when correct key/fob disarms the system and engine starts.</t>
+        </is>
+      </c>
+      <c r="N30" s="3" t="inlineStr"/>
+    </row>
+    <row r="31" ht="100" customHeight="1">
+      <c r="A31" s="4" t="inlineStr"/>
+      <c r="B31" s="5" t="inlineStr">
+        <is>
+          <t>4WD / AWD Engaged</t>
+        </is>
+      </c>
+      <c r="C31" s="5" t="inlineStr">
+        <is>
+          <t>Direct – FMVSS 101, Table 2 (voluntary)</t>
+        </is>
+      </c>
+      <c r="D31" s="5" t="inlineStr">
+        <is>
+          <t>UN R121, Table 1</t>
+        </is>
+      </c>
+      <c r="E31" s="5" t="inlineStr"/>
+      <c r="F31" s="5" t="inlineStr">
+        <is>
+          <t>ISO 2575:2021, Symbol 7000-0791</t>
+        </is>
+      </c>
+      <c r="G31" s="5" t="inlineStr">
+        <is>
+          <t>ISO 2575:2021 Cl. 5.2: minimum symbol height 5 mm at design eye point. SAE J1005: symbol ≥3.2 mm; text/numerals ≥4.8 mm. FMVSS 101 S5.3: legible at 76 cm viewing distance.</t>
+        </is>
+      </c>
+      <c r="H31" s="5" t="inlineStr">
+        <is>
+          <t>Green (engaged) or Amber (fault)</t>
+        </is>
+      </c>
+      <c r="I31" s="5" t="inlineStr">
+        <is>
+          <t>Text '4WD', '4×4', 'AWD', or four-wheel silhouette. Green indicates normal 4WD/AWD engagement; amber indicates a system fault. OEM nomenclature varies.</t>
+        </is>
+      </c>
+      <c r="J31" s="5" t="inlineStr">
+        <is>
+          <t>SAE J387 / ECE R121 Annex 4: minimum luminance 2 cd/m² (night), max 100 cd/m² (to prevent glare). Daytime: 100–1 000 cd/m².</t>
+        </is>
+      </c>
+      <c r="K31" s="5" t="inlineStr">
+        <is>
+          <t>SAE J2402: ≥3:1 luminance contrast during day; ≥4.5:1 during night. Symbol-to-background ratio.</t>
+        </is>
+      </c>
+      <c r="L31" s="5" t="inlineStr">
+        <is>
+          <t>Within the driver's primary field of view (FMVSS 101 S5.1). Visible without head movement. Not obscured by steering wheel.</t>
+        </is>
+      </c>
+      <c r="M31" s="5" t="inlineStr">
+        <is>
+          <t>GREEN: 4WD or AWD system is actively engaged. Illuminates when driver selects 4H or 4L range (part-time 4WD), or when AWD coupling is engaged. Extinguishes when 2WD is selected or AWD decouples. AMBER: 4WD/AWD system fault; requires service.</t>
+        </is>
+      </c>
+      <c r="N31" s="5" t="inlineStr">
+        <is>
+          <t>FWD/RWD-only vehicles without selectable 4WD/AWD.</t>
+        </is>
+      </c>
+    </row>
+    <row r="32" ht="100" customHeight="1">
+      <c r="A32" s="2" t="inlineStr"/>
+      <c r="B32" s="3" t="inlineStr">
+        <is>
+          <t>Differential Lock Engaged</t>
+        </is>
+      </c>
+      <c r="C32" s="3" t="inlineStr">
+        <is>
+          <t>Direct – FMVSS 101, Table 2 (voluntary)</t>
+        </is>
+      </c>
+      <c r="D32" s="3" t="inlineStr">
+        <is>
+          <t>UN R121, Table 1</t>
+        </is>
+      </c>
+      <c r="E32" s="3" t="inlineStr"/>
+      <c r="F32" s="3" t="inlineStr">
+        <is>
+          <t>ISO 2575:2021, Symbol 7000-0790</t>
+        </is>
+      </c>
+      <c r="G32" s="3" t="inlineStr">
+        <is>
+          <t>ISO 2575:2021 Cl. 5.2: minimum symbol height 5 mm at design eye point. SAE J1005: symbol ≥3.2 mm; text/numerals ≥4.8 mm. FMVSS 101 S5.3: legible at 76 cm viewing distance.</t>
+        </is>
+      </c>
+      <c r="H32" s="3" t="inlineStr">
+        <is>
+          <t>Amber (engaging/fault) or Green (fully locked)</t>
+        </is>
+      </c>
+      <c r="I32" s="3" t="inlineStr">
+        <is>
+          <t>Symbol showing rear axle with lock indicator. Text 'DIFF LOCK' may be used. OEM practice varies; some use amber for lock-in-progress and green for fully locked.</t>
+        </is>
+      </c>
+      <c r="J32" s="3" t="inlineStr">
+        <is>
+          <t>SAE J387 / ECE R121 Annex 4: minimum luminance 2 cd/m² (night), max 100 cd/m² (to prevent glare). Daytime: 100–1 000 cd/m².</t>
+        </is>
+      </c>
+      <c r="K32" s="3" t="inlineStr">
+        <is>
+          <t>SAE J2402: ≥3:1 luminance contrast during day; ≥4.5:1 during night. Symbol-to-background ratio.</t>
+        </is>
+      </c>
+      <c r="L32" s="3" t="inlineStr">
+        <is>
+          <t>Within the driver's primary field of view (FMVSS 101 S5.1). Visible without head movement. Not obscured by steering wheel.</t>
+        </is>
+      </c>
+      <c r="M32" s="3" t="inlineStr">
+        <is>
+          <t>Illuminates while the differential lock is being engaged (amber/flashing) and when fully locked (steady green or amber depending on OEM). Extinguishes when differential unlocks. Locking/unlocking typically requires vehicle speed &lt; ~8 km/h.</t>
+        </is>
+      </c>
+      <c r="N32" s="3" t="inlineStr">
+        <is>
+          <t>Vehicles without differential lock mechanism.</t>
+        </is>
+      </c>
+    </row>
+    <row r="33" ht="100" customHeight="1">
+      <c r="A33" s="4" t="inlineStr"/>
+      <c r="B33" s="5" t="inlineStr">
+        <is>
+          <t>Cruise Control Active</t>
+        </is>
+      </c>
+      <c r="C33" s="5" t="inlineStr">
+        <is>
+          <t>Direct – FMVSS 101, Table 2 (voluntary)
+Indirect – SAE J1359 (cruise control)</t>
+        </is>
+      </c>
+      <c r="D33" s="5" t="inlineStr">
+        <is>
+          <t>UN R121, Table 1</t>
+        </is>
+      </c>
+      <c r="E33" s="5" t="inlineStr"/>
+      <c r="F33" s="5" t="inlineStr">
+        <is>
+          <t>ISO 2575:2021, Symbol 7000-0482</t>
+        </is>
+      </c>
+      <c r="G33" s="5" t="inlineStr">
+        <is>
+          <t>ISO 2575:2021 Cl. 5.2: minimum symbol height 5 mm at design eye point. SAE J1005: symbol ≥3.2 mm; text/numerals ≥4.8 mm. FMVSS 101 S5.3: legible at 76 cm viewing distance.</t>
+        </is>
+      </c>
+      <c r="H33" s="5" t="inlineStr">
+        <is>
+          <t>Green</t>
+        </is>
+      </c>
+      <c r="I33" s="5" t="inlineStr">
+        <is>
+          <t>Speedometer arc with SET indicator or text 'CRUISE'. Green = system is set and actively controlling speed.</t>
+        </is>
+      </c>
+      <c r="J33" s="5" t="inlineStr">
+        <is>
+          <t>SAE J387 / ECE R121 Annex 4: minimum luminance 2 cd/m² (night), max 100 cd/m² (to prevent glare). Daytime: 100–1 000 cd/m².</t>
+        </is>
+      </c>
+      <c r="K33" s="5" t="inlineStr">
+        <is>
+          <t>SAE J2402: ≥3:1 luminance contrast during day; ≥4.5:1 during night. Symbol-to-background ratio.</t>
+        </is>
+      </c>
+      <c r="L33" s="5" t="inlineStr">
+        <is>
+          <t>Within the driver's primary field of view (FMVSS 101 S5.1). Visible without head movement. Not obscured by steering wheel.</t>
+        </is>
+      </c>
+      <c r="M33" s="5" t="inlineStr">
+        <is>
+          <t>Illuminates when conventional cruise control is set and actively maintaining the set speed. Extinguishes when cruise is cancelled (brake/clutch press, manual cancel) or when speed falls outside controllable range.</t>
+        </is>
+      </c>
+      <c r="N33" s="5" t="inlineStr"/>
+    </row>
+    <row r="34" ht="100" customHeight="1">
+      <c r="A34" s="2" t="inlineStr"/>
+      <c r="B34" s="3" t="inlineStr">
+        <is>
+          <t>Adaptive Cruise Control (ACC) Active</t>
+        </is>
+      </c>
+      <c r="C34" s="3" t="inlineStr">
+        <is>
+          <t>Direct – FMVSS 101, Table 2 (voluntary)
+Indirect – SAE J3048 (ACC)</t>
+        </is>
+      </c>
+      <c r="D34" s="3" t="inlineStr">
+        <is>
+          <t>UN R131 (advanced emergency braking)
+UN R121</t>
+        </is>
+      </c>
+      <c r="E34" s="3" t="inlineStr"/>
+      <c r="F34" s="3" t="inlineStr">
+        <is>
+          <t>ISO 2575:2021, Symbol 7000-2427</t>
+        </is>
+      </c>
+      <c r="G34" s="3" t="inlineStr">
+        <is>
+          <t>ISO 2575:2021 Cl. 5.2: minimum symbol height 5 mm at design eye point. SAE J1005: symbol ≥3.2 mm; text/numerals ≥4.8 mm. FMVSS 101 S5.3: legible at 76 cm viewing distance.</t>
+        </is>
+      </c>
+      <c r="H34" s="3" t="inlineStr">
+        <is>
+          <t>Green (active / following) or Amber (standby/fault)</t>
+        </is>
+      </c>
+      <c r="I34" s="3" t="inlineStr">
+        <is>
+          <t>Lead vehicle outline with arcs (radar) plus own vehicle symbol and SET/speed indicator. Green = actively following or holding set speed. Amber = ACC in standby or fault.</t>
+        </is>
+      </c>
+      <c r="J34" s="3" t="inlineStr">
+        <is>
+          <t>SAE J387 / ECE R121 Annex 4: minimum luminance 2 cd/m² (night), max 100 cd/m² (to prevent glare). Daytime: 100–1 000 cd/m².</t>
+        </is>
+      </c>
+      <c r="K34" s="3" t="inlineStr">
+        <is>
+          <t>SAE J2402: ≥3:1 luminance contrast during day; ≥4.5:1 during night. Symbol-to-background ratio.</t>
+        </is>
+      </c>
+      <c r="L34" s="3" t="inlineStr">
+        <is>
+          <t>Within the driver's primary field of view (FMVSS 101 S5.1). Visible without head movement. Not obscured by steering wheel.</t>
+        </is>
+      </c>
+      <c r="M34" s="3" t="inlineStr">
+        <is>
+          <t>GREEN: ACC is active and controlling speed/following distance. FLASHING GREEN: ACC braking event occurring. AMBER (steady): ACC standby (below minimum speed or system detecting too many cut-ins). AMBER (flashing / steady): ACC malfunction, requires service.</t>
+        </is>
+      </c>
+      <c r="N34" s="3" t="inlineStr">
+        <is>
+          <t>Vehicles not equipped with ACC radar sensor.</t>
+        </is>
+      </c>
+    </row>
+    <row r="35" ht="100" customHeight="1">
+      <c r="A35" s="4" t="inlineStr"/>
+      <c r="B35" s="5" t="inlineStr">
+        <is>
+          <t>Lane Departure Warning (LDW)</t>
+        </is>
+      </c>
+      <c r="C35" s="5" t="inlineStr">
+        <is>
+          <t>Direct – FMVSS 101, Table 2 (voluntary)
+Indirect – NHTSA FMVSS 126 (references ESC; no dedicated FMVSS for LDW in US as of 2024)</t>
+        </is>
+      </c>
+      <c r="D35" s="5" t="inlineStr">
+        <is>
+          <t>UN R130 (lane departure warning systems)
+UN R121</t>
+        </is>
+      </c>
+      <c r="E35" s="5" t="inlineStr"/>
+      <c r="F35" s="5" t="inlineStr">
+        <is>
+          <t>ISO 2575:2021, Symbol 7000-2548</t>
+        </is>
+      </c>
+      <c r="G35" s="5" t="inlineStr">
+        <is>
+          <t>ISO 2575:2021 Cl. 5.2: minimum symbol height 5 mm at design eye point. SAE J1005: symbol ≥3.2 mm; text/numerals ≥4.8 mm. FMVSS 101 S5.3: legible at 76 cm viewing distance.</t>
+        </is>
+      </c>
+      <c r="H35" s="5" t="inlineStr">
+        <is>
+          <t>Amber (warning) or Green (system on, no warning)</t>
+        </is>
+      </c>
+      <c r="I35" s="5" t="inlineStr">
+        <is>
+          <t>Top-view vehicle between two lane lines, with one line highlighted or pulsing to indicate departure side. Green version: system active and monitoring. Amber: active warning of lane departure.</t>
+        </is>
+      </c>
+      <c r="J35" s="5" t="inlineStr">
+        <is>
+          <t>SAE J387 / ECE R121 Annex 4: minimum luminance 2 cd/m² (night), max 100 cd/m² (to prevent glare). Daytime: 100–1 000 cd/m².</t>
+        </is>
+      </c>
+      <c r="K35" s="5" t="inlineStr">
+        <is>
+          <t>SAE J2402: ≥3:1 luminance contrast during day; ≥4.5:1 during night. Symbol-to-background ratio.</t>
+        </is>
+      </c>
+      <c r="L35" s="5" t="inlineStr">
+        <is>
+          <t>Within the driver's primary field of view (FMVSS 101 S5.1). Visible without head movement. Not obscured by steering wheel.</t>
+        </is>
+      </c>
+      <c r="M35" s="5" t="inlineStr">
+        <is>
+          <t>GREEN: LDW system is on and monitoring lane markings. AMBER (flashing): unintentional lane crossing detected (no turn signal active). Warning ceases when driver steers back or activates turn signal. AMBER (steady): LDW system fault or camera obstructed. UN R130 specifies timing constraints for the warning.</t>
+        </is>
+      </c>
+      <c r="N35" s="5" t="inlineStr"/>
+    </row>
+    <row r="36" ht="100" customHeight="1">
+      <c r="A36" s="2" t="inlineStr"/>
+      <c r="B36" s="3" t="inlineStr">
+        <is>
+          <t>Forward Collision Warning (FCW)</t>
+        </is>
+      </c>
+      <c r="C36" s="3" t="inlineStr">
+        <is>
+          <t>Direct – FMVSS 101, Table 2 (voluntary)
+Indirect – NHTSA NCAP encourages FCW but no dedicated FMVSS as of 2024</t>
+        </is>
+      </c>
+      <c r="D36" s="3" t="inlineStr">
+        <is>
+          <t>UN R152 (advanced emergency braking)
+UN R121</t>
+        </is>
+      </c>
+      <c r="E36" s="3" t="inlineStr"/>
+      <c r="F36" s="3" t="inlineStr">
+        <is>
+          <t>ISO 2575:2021, Symbol 7000-2549</t>
+        </is>
+      </c>
+      <c r="G36" s="3" t="inlineStr">
+        <is>
+          <t>ISO 2575:2021 Cl. 5.2: minimum symbol height 5 mm at design eye point. SAE J1005: symbol ≥3.2 mm; text/numerals ≥4.8 mm. FMVSS 101 S5.3: legible at 76 cm viewing distance.</t>
+        </is>
+      </c>
+      <c r="H36" s="3" t="inlineStr">
+        <is>
+          <t>Amber (warning) or Red (imminent collision)</t>
+        </is>
+      </c>
+      <c r="I36" s="3" t="inlineStr">
+        <is>
+          <t>Two vehicle silhouettes (lead and host) with collision alert symbol or exclamation marks between them. Amber for time-to-collision warning; red for imminent-collision alert.</t>
+        </is>
+      </c>
+      <c r="J36" s="3" t="inlineStr">
+        <is>
+          <t>SAE J387 / ECE R121 Annex 4: minimum luminance 2 cd/m² (night), max 100 cd/m² (to prevent glare). Daytime: 100–1 000 cd/m².</t>
+        </is>
+      </c>
+      <c r="K36" s="3" t="inlineStr">
+        <is>
+          <t>SAE J2402: ≥3:1 luminance contrast during day; ≥4.5:1 during night. Symbol-to-background ratio.</t>
+        </is>
+      </c>
+      <c r="L36" s="3" t="inlineStr">
+        <is>
+          <t>Within the driver's primary field of view (FMVSS 101 S5.1). Visible without head movement. Not obscured by steering wheel.</t>
+        </is>
+      </c>
+      <c r="M36" s="3" t="inlineStr">
+        <is>
+          <t>AMBER: vehicle ahead detected with insufficient following distance at current speed; driver alert required. RED (if equipped): collision imminent; AEB may activate. Extinguishes when adequate following distance is restored or AEB intervenes. Audible chime accompanies visual warning.</t>
+        </is>
+      </c>
+      <c r="N36" s="3" t="inlineStr"/>
+    </row>
+    <row r="37" ht="100" customHeight="1">
+      <c r="A37" s="4" t="inlineStr"/>
+      <c r="B37" s="5" t="inlineStr">
+        <is>
+          <t>Blind Spot Information / Warning</t>
+        </is>
+      </c>
+      <c r="C37" s="5" t="inlineStr">
+        <is>
+          <t>Direct – FMVSS 101, Table 2 (voluntary)
+Indirect – NHTSA FMVSS 111 (rear visibility); no dedicated FMVSS for BSD as of 2024</t>
+        </is>
+      </c>
+      <c r="D37" s="5" t="inlineStr">
+        <is>
+          <t>UN R151 (blind spot information systems)
+UN R121</t>
+        </is>
+      </c>
+      <c r="E37" s="5" t="inlineStr"/>
+      <c r="F37" s="5" t="inlineStr">
+        <is>
+          <t>ISO 2575:2021, Symbol 7000-2509</t>
+        </is>
+      </c>
+      <c r="G37" s="5" t="inlineStr">
+        <is>
+          <t>ISO 2575:2021 Cl. 5.2: minimum symbol height 5 mm at design eye point. SAE J1005: symbol ≥3.2 mm; text/numerals ≥4.8 mm. FMVSS 101 S5.3: legible at 76 cm viewing distance.</t>
+        </is>
+      </c>
+      <c r="H37" s="5" t="inlineStr">
+        <is>
+          <t>Amber</t>
+        </is>
+      </c>
+      <c r="I37" s="5" t="inlineStr">
+        <is>
+          <t>Top-view vehicle with triangular zone or car icon in adjacent lane highlighted amber. Typically displayed in or near the door mirror on the warning side.</t>
+        </is>
+      </c>
+      <c r="J37" s="5" t="inlineStr">
+        <is>
+          <t>SAE J387 / ECE R121 Annex 4: minimum luminance 2 cd/m² (night), max 100 cd/m² (to prevent glare). Daytime: 100–1 000 cd/m².</t>
+        </is>
+      </c>
+      <c r="K37" s="5" t="inlineStr">
+        <is>
+          <t>SAE J2402: ≥3:1 luminance contrast during day; ≥4.5:1 during night. Symbol-to-background ratio.</t>
+        </is>
+      </c>
+      <c r="L37" s="5" t="inlineStr">
+        <is>
+          <t>Within the driver's primary field of view (FMVSS 101 S5.1). Visible without head movement. Not obscured by steering wheel.</t>
+        </is>
+      </c>
+      <c r="M37" s="5" t="inlineStr">
+        <is>
+          <t>Illuminates (amber) in the relevant mirror or A-pillar area when an object (vehicle) is detected in the blind zone alongside the host vehicle. If driver activates turn signal while object is detected, telltale flashes rapidly (urgent warning). Extinguishes when the lane is clear. UN R151 defines detection zone geometry.</t>
+        </is>
+      </c>
+      <c r="N37" s="5" t="inlineStr"/>
+    </row>
+    <row r="38" ht="100" customHeight="1">
+      <c r="A38" s="2" t="inlineStr"/>
+      <c r="B38" s="3" t="inlineStr">
+        <is>
+          <t>Speed Limiter Active</t>
+        </is>
+      </c>
+      <c r="C38" s="3" t="inlineStr">
+        <is>
+          <t>Direct – FMVSS 101, Table 2 (voluntary)</t>
+        </is>
+      </c>
+      <c r="D38" s="3" t="inlineStr">
+        <is>
+          <t>UN R65 (speed limitation devices)
+UN R121</t>
+        </is>
+      </c>
+      <c r="E38" s="3" t="inlineStr">
+        <is>
+          <t>ECE R65</t>
+        </is>
+      </c>
+      <c r="F38" s="3" t="inlineStr">
+        <is>
+          <t>ISO 2575:2021, Symbol 7000-2462</t>
+        </is>
+      </c>
+      <c r="G38" s="3" t="inlineStr">
+        <is>
+          <t>ISO 2575:2021 Cl. 5.2: minimum symbol height 5 mm at design eye point. SAE J1005: symbol ≥3.2 mm; text/numerals ≥4.8 mm. FMVSS 101 S5.3: legible at 76 cm viewing distance.</t>
+        </is>
+      </c>
+      <c r="H38" s="3" t="inlineStr">
+        <is>
+          <t>Amber (active) or Red (fault)</t>
+        </is>
+      </c>
+      <c r="I38" s="3" t="inlineStr">
+        <is>
+          <t>Speedometer circle with a horizontal line indicating a cap, plus speed value or 'LIM' text. Amber = actively limiting. Red = system fault.</t>
+        </is>
+      </c>
+      <c r="J38" s="3" t="inlineStr">
+        <is>
+          <t>SAE J387 / ECE R121 Annex 4: minimum luminance 2 cd/m² (night), max 100 cd/m² (to prevent glare). Daytime: 100–1 000 cd/m².</t>
+        </is>
+      </c>
+      <c r="K38" s="3" t="inlineStr">
+        <is>
+          <t>SAE J2402: ≥3:1 luminance contrast during day; ≥4.5:1 during night. Symbol-to-background ratio.</t>
+        </is>
+      </c>
+      <c r="L38" s="3" t="inlineStr">
+        <is>
+          <t>Within the driver's primary field of view (FMVSS 101 S5.1). Visible without head movement. Not obscured by steering wheel.</t>
+        </is>
+      </c>
+      <c r="M38" s="3" t="inlineStr">
+        <is>
+          <t>AMBER: vehicle's speed limiter is engaged and preventing acceleration above the set speed. Extinguishes when the limiter is cancelled or overridden. RED: speed limiter malfunction; UN R65 requires the driver to be alerted to system failure.</t>
+        </is>
+      </c>
+      <c r="N38" s="3" t="inlineStr"/>
+    </row>
+    <row r="39" ht="100" customHeight="1">
+      <c r="A39" s="4" t="inlineStr"/>
+      <c r="B39" s="5" t="inlineStr">
+        <is>
+          <t>Electric Powertrain Ready (EV / HEV)</t>
+        </is>
+      </c>
+      <c r="C39" s="5" t="inlineStr">
+        <is>
+          <t>Direct – FMVSS 101, Table 2 (voluntary)
+Indirect – SAE J3068, FMVSS 305 (electric vehicle safety)</t>
+        </is>
+      </c>
+      <c r="D39" s="5" t="inlineStr">
+        <is>
+          <t>UN R100 (electric vehicle safety)
+UN R121</t>
+        </is>
+      </c>
+      <c r="E39" s="5" t="inlineStr">
+        <is>
+          <t>ECE R100</t>
+        </is>
+      </c>
+      <c r="F39" s="5" t="inlineStr">
+        <is>
+          <t>ISO 2575:2021, Symbol 7000-2378</t>
+        </is>
+      </c>
+      <c r="G39" s="5" t="inlineStr">
+        <is>
+          <t>ISO 2575:2021 Cl. 5.2: minimum symbol height 5 mm at design eye point. SAE J1005: symbol ≥3.2 mm; text/numerals ≥4.8 mm. FMVSS 101 S5.3: legible at 76 cm viewing distance.</t>
+        </is>
+      </c>
+      <c r="H39" s="5" t="inlineStr">
+        <is>
+          <t>Green</t>
+        </is>
+      </c>
+      <c r="I39" s="5" t="inlineStr">
+        <is>
+          <t>Text 'READY' or EV powertrain symbol (e.g., plug with leaf/lightning bolt). Green = vehicle is in a driveable state (power train energised).</t>
+        </is>
+      </c>
+      <c r="J39" s="5" t="inlineStr">
+        <is>
+          <t>SAE J387 / ECE R121 Annex 4: minimum luminance 2 cd/m² (night), max 100 cd/m² (to prevent glare). Daytime: 100–1 000 cd/m².</t>
+        </is>
+      </c>
+      <c r="K39" s="5" t="inlineStr">
+        <is>
+          <t>SAE J2402: ≥3:1 luminance contrast during day; ≥4.5:1 during night. Symbol-to-background ratio.</t>
+        </is>
+      </c>
+      <c r="L39" s="5" t="inlineStr">
+        <is>
+          <t>Within the driver's primary field of view (FMVSS 101 S5.1). Visible without head movement. Not obscured by steering wheel.</t>
+        </is>
+      </c>
+      <c r="M39" s="5" t="inlineStr">
+        <is>
+          <t>Illuminates when the electric drive system is fully powered and the vehicle is ready to move. Extinguishes when ignition/power is turned off or vehicle is placed in park and de-energised. Absence of this telltale in an EV indicates the vehicle is NOT driveable.</t>
+        </is>
+      </c>
+      <c r="N39" s="5" t="inlineStr">
+        <is>
+          <t>Conventional ICE-only vehicles without EV/HEV powertrain.</t>
+        </is>
+      </c>
+    </row>
+    <row r="40" ht="100" customHeight="1">
+      <c r="A40" s="2" t="inlineStr"/>
+      <c r="B40" s="3" t="inlineStr">
+        <is>
+          <t>High-Voltage Battery Low (EV / HEV)</t>
+        </is>
+      </c>
+      <c r="C40" s="3" t="inlineStr">
+        <is>
+          <t>Direct – FMVSS 101, Table 2 (voluntary)
+Indirect – FMVSS 305 (electric vehicle energy storage)</t>
+        </is>
+      </c>
+      <c r="D40" s="3" t="inlineStr">
+        <is>
+          <t>UN R100 (electric vehicle safety)
+UN R121</t>
+        </is>
+      </c>
+      <c r="E40" s="3" t="inlineStr">
+        <is>
+          <t>ECE R100</t>
+        </is>
+      </c>
+      <c r="F40" s="3" t="inlineStr">
+        <is>
+          <t>ISO 2575:2021, Symbol 7000-2379</t>
+        </is>
+      </c>
+      <c r="G40" s="3" t="inlineStr">
+        <is>
+          <t>ISO 2575:2021 Cl. 5.2: minimum symbol height 5 mm at design eye point. SAE J1005: symbol ≥3.2 mm; text/numerals ≥4.8 mm. FMVSS 101 S5.3: legible at 76 cm viewing distance.</t>
+        </is>
+      </c>
+      <c r="H40" s="3" t="inlineStr">
+        <is>
+          <t>Amber (low state-of-charge) or Red (critically low)</t>
+        </is>
+      </c>
+      <c r="I40" s="3" t="inlineStr">
+        <is>
+          <t>Battery symbol (HV battery shape) with low fill indicator and exclamation mark or downward arrow. Must be visually distinct from the 12 V battery/charging telltale.</t>
+        </is>
+      </c>
+      <c r="J40" s="3" t="inlineStr">
+        <is>
+          <t>SAE J387 / ECE R121 Annex 4: minimum luminance 2 cd/m² (night), max 100 cd/m² (to prevent glare). Daytime: 100–1 000 cd/m².</t>
+        </is>
+      </c>
+      <c r="K40" s="3" t="inlineStr">
+        <is>
+          <t>SAE J2402: ≥3:1 luminance contrast during day; ≥4.5:1 during night. Symbol-to-background ratio.</t>
+        </is>
+      </c>
+      <c r="L40" s="3" t="inlineStr">
+        <is>
+          <t>Within the driver's primary field of view (FMVSS 101 S5.1). Visible without head movement. Not obscured by steering wheel.</t>
+        </is>
+      </c>
+      <c r="M40" s="3" t="inlineStr">
+        <is>
+          <t>AMBER: high-voltage traction battery state-of-charge has fallen below the OEM low-charge threshold (typically ~10–15 % SoC remaining). Driver must recharge promptly. RED: critical charge level; range may be severely limited. Extinguishes when battery is charged above the threshold.</t>
+        </is>
+      </c>
+      <c r="N40" s="3" t="inlineStr">
+        <is>
+          <t>Conventional ICE-only vehicles.</t>
+        </is>
+      </c>
+    </row>
+    <row r="41" ht="100" customHeight="1">
+      <c r="A41" s="4" t="inlineStr"/>
+      <c r="B41" s="5" t="inlineStr">
+        <is>
+          <t>EV Charging Active / Connected</t>
+        </is>
+      </c>
+      <c r="C41" s="5" t="inlineStr">
+        <is>
+          <t>Direct – FMVSS 101, Table 2 (voluntary)
+Indirect – SAE J1772 (EV charging connector); FMVSS 305</t>
+        </is>
+      </c>
+      <c r="D41" s="5" t="inlineStr">
+        <is>
+          <t>UN R100
+UN R121</t>
+        </is>
+      </c>
+      <c r="E41" s="5" t="inlineStr">
+        <is>
+          <t>ECE R100</t>
+        </is>
+      </c>
+      <c r="F41" s="5" t="inlineStr">
+        <is>
+          <t>ISO 2575:2021, Symbol 7000-2380</t>
+        </is>
+      </c>
+      <c r="G41" s="5" t="inlineStr">
+        <is>
+          <t>ISO 2575:2021 Cl. 5.2: minimum symbol height 5 mm at design eye point. SAE J1005: symbol ≥3.2 mm; text/numerals ≥4.8 mm. FMVSS 101 S5.3: legible at 76 cm viewing distance.</t>
+        </is>
+      </c>
+      <c r="H41" s="5" t="inlineStr">
+        <is>
+          <t>Green (charging normally) or Amber (fault/incomplete)</t>
+        </is>
+      </c>
+      <c r="I41" s="5" t="inlineStr">
+        <is>
+          <t>Plug symbol with lightning bolt or battery charging indicator. Green = charging in progress or complete. Amber = charging fault, cable not fully connected, or wrong power supply.</t>
+        </is>
+      </c>
+      <c r="J41" s="5" t="inlineStr">
+        <is>
+          <t>SAE J387 / ECE R121 Annex 4: minimum luminance 2 cd/m² (night), max 100 cd/m² (to prevent glare). Daytime: 100–1 000 cd/m².</t>
+        </is>
+      </c>
+      <c r="K41" s="5" t="inlineStr">
+        <is>
+          <t>SAE J2402: ≥3:1 luminance contrast during day; ≥4.5:1 during night. Symbol-to-background ratio.</t>
+        </is>
+      </c>
+      <c r="L41" s="5" t="inlineStr">
+        <is>
+          <t>Within the driver's primary field of view (FMVSS 101 S5.1). Visible without head movement. Not obscured by steering wheel.</t>
+        </is>
+      </c>
+      <c r="M41" s="5" t="inlineStr">
+        <is>
+          <t>GREEN: EVSE connected and charging is proceeding normally. May pulse/animate to indicate charging in progress. STEADY GREEN: charge complete. AMBER: charging interrupted or fault (thermal event, EVSE incompatibility, ground fault). SAE J1772 defines signal protocol between EVSE and vehicle. Extinguishes when cable is disconnected and vehicle is powered on.</t>
+        </is>
+      </c>
+      <c r="N41" s="5" t="inlineStr">
+        <is>
+          <t>Conventional ICE-only vehicles.</t>
+        </is>
+      </c>
+    </row>
+    <row r="43" ht="20" customHeight="1">
+      <c r="A43" s="6" t="inlineStr">
+        <is>
+          <t>SOURCES: 49 CFR 571.101 (FMVSS 101) · FMVSS 105/108/121/126/135/136/138/208 · UN ECE R13/R13H/R16/R48/R55/R65/R83/R94/R100/R116/R121/R130/R131/R139/R140/R141/R151/R152 · ISO 2575:2021 (Symbols) · SAE J387 · SAE J1005 · SAE J2402 · SAE J1979 (OBD-II)</t>
+        </is>
+      </c>
+    </row>
+    <row r="44" ht="16" customHeight="1">
+      <c r="A44" s="6" t="inlineStr">
+        <is>
+          <t>Color key: 🔴 Red = immediate safety hazard, stop vehicle  🟡 Amber = attention/service required  🟢 Green = normal operational status  🔵 Blue = informational (high beam)</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <mergeCells count="1">
-    <mergeCell ref="A15:N15"/>
+  <mergeCells count="2">
+    <mergeCell ref="A43:N43"/>
+    <mergeCell ref="A44:N44"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>

</xml_diff>